<commit_message>
Updated spreadsheet with 63 websites, 64 phones - 28% complete
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -732,6 +732,11 @@
           <ns0:t>(781) 686-5049</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>accounts@vaughanplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F15" t="inlineStr">
         <ns0:is>
           <ns0:t>Boston, MA</ns0:t>
@@ -745,6 +750,11 @@
       <ns0:c r="I15" t="inlineStr">
         <ns0:is>
           <ns0:t>YES (100+ yrs)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J15" t="inlineStr">
+        <ns0:is>
+          <ns0:t>vaughanplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K15" t="inlineStr">
@@ -791,7 +801,7 @@
       </ns0:c>
       <ns0:c r="J16" t="inlineStr">
         <ns0:is>
-          <ns0:t>rotorooter.com</ns0:t>
+          <ns0:t>serviceplusplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K16" t="inlineStr">
@@ -821,6 +831,11 @@
           <ns0:t>(615) 205-7656</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jonathan@loftyrankings.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
           <ns0:t>3744 Annex Ave</ns0:t>
@@ -838,7 +853,7 @@
       </ns0:c>
       <ns0:c r="J17" t="inlineStr">
         <ns0:is>
-          <ns0:t>benchmarkplumbingtn.com</ns0:t>
+          <ns0:t>southernplumbingworks.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K17" t="inlineStr">
@@ -883,6 +898,11 @@
           <ns0:t>YES (family)</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J18" t="inlineStr">
+        <ns0:is>
+          <ns0:t>wyattworksplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K18" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -927,7 +947,7 @@
       </ns0:c>
       <ns0:c r="J19" t="inlineStr">
         <ns0:is>
-          <ns0:t>ericasplumbing.com</ns0:t>
+          <ns0:t>miamidadeplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K19" t="inlineStr">
@@ -974,7 +994,7 @@
       </ns0:c>
       <ns0:c r="J20" t="inlineStr">
         <ns0:is>
-          <ns0:t>radiantplumbingga.com</ns0:t>
+          <ns0:t>headsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K20" t="inlineStr">
@@ -1021,7 +1041,7 @@
       </ns0:c>
       <ns0:c r="J21" t="inlineStr">
         <ns0:is>
-          <ns0:t>rotorooter.com</ns0:t>
+          <ns0:t>halpinplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K21" t="inlineStr">
@@ -1066,6 +1086,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J22" t="inlineStr">
+        <ns0:is>
+          <ns0:t>stinenichols.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K22" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1229,6 +1254,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J26" t="inlineStr">
+        <ns0:is>
+          <ns0:t>allstarplumbingfresno.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K26" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1256,6 +1286,11 @@
           <ns0:t>(520) 850-4552</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>impallari@gmail.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
           <ns0:t>1665 E 18th St #117</ns0:t>
@@ -1269,6 +1304,11 @@
       <ns0:c r="I27" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J27" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jobeandsonsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K27" t="inlineStr">
@@ -1298,6 +1338,11 @@
           <ns0:t>(562) 459-6445</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>info@thefamilyplumber.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
           <ns0:t>3613 Briggeman Dr</ns0:t>
@@ -1311,6 +1356,11 @@
       <ns0:c r="I28" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J28" t="inlineStr">
+        <ns0:is>
+          <ns0:t>thefamilyplumber.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K28" t="inlineStr">
@@ -1355,6 +1405,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J29" t="inlineStr">
+        <ns0:is>
+          <ns0:t>armstrongplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K29" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1397,6 +1452,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J30" t="inlineStr">
+        <ns0:is>
+          <ns0:t>williamparrishplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K30" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1424,6 +1484,11 @@
           <ns0:t>(813) 443-5820</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>info@olinplumbinginc.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
           <ns0:t>3201 E 8th Ave</ns0:t>
@@ -1437,6 +1502,11 @@
       <ns0:c r="I31" t="inlineStr">
         <ns0:is>
           <ns0:t>YES (family)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J31" t="inlineStr">
+        <ns0:is>
+          <ns0:t>olinplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K31" t="inlineStr">
@@ -1575,6 +1645,11 @@
           <ns0:t>YES (1959)</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J34" t="inlineStr">
+        <ns0:is>
+          <ns0:t>lyonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K34" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1617,6 +1692,11 @@
           <ns0:t>YES (1985)</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J35" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jjsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K35" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1659,6 +1739,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J36" t="inlineStr">
+        <ns0:is>
+          <ns0:t>allstarplumbingfresno.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K36" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -1686,6 +1771,11 @@
           <ns0:t>(520) 850-4552</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>impallari@gmail.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
           <ns0:t>1665 E 18th St #117</ns0:t>
@@ -1699,6 +1789,11 @@
       <ns0:c r="I37" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J37" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jobeandsonsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K37" t="inlineStr">
@@ -1812,6 +1907,11 @@
           <ns0:t>(817) 819-1471</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>e7d54b729aaf49ea8b2f80dae22860aa@sentry.zipify.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F40" t="inlineStr">
         <ns0:is>
           <ns0:t>Arlington, TX</ns0:t>
@@ -1825,6 +1925,11 @@
       <ns0:c r="I40" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J40" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familyfriends.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K40" t="inlineStr">
@@ -2007,6 +2112,11 @@
           <ns0:t>(314) 965-9377</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E45" t="inlineStr">
+        <ns0:is>
+          <ns0:t>pl_a_055-300x200@2x.jpeg</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
           <ns0:t>5705 Dale Ave</ns0:t>
@@ -2020,6 +2130,11 @@
       <ns0:c r="I45" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J45" t="inlineStr">
+        <ns0:is>
+          <ns0:t>tonylamartinaplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K45" t="inlineStr">
@@ -2091,6 +2206,11 @@
           <ns0:t>(361) 241-6000</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E47" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mccainplumbing@sbcglobal.net</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
           <ns0:t>9725 Leopard St</ns0:t>
@@ -2104,6 +2224,11 @@
       <ns0:c r="I47" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J47" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dwainmccainplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K47" t="inlineStr">
@@ -2148,6 +2273,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J48" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dauenhauerplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K48" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2190,6 +2320,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J49" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robinsonfamilyplumbinghvac.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K49" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2232,6 +2367,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J50" t="inlineStr">
+        <ns0:is>
+          <ns0:t>barkerandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K50" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2306,6 +2446,11 @@
           <ns0:t>(657) 229-2993</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E52" t="inlineStr">
+        <ns0:is>
+          <ns0:t>leads@doitrightplumbers.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
           <ns0:t>1630 Palm St</ns0:t>
@@ -2319,6 +2464,11 @@
       <ns0:c r="I52" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J52" t="inlineStr">
+        <ns0:is>
+          <ns0:t>doitrightplumbers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K52" t="inlineStr">
@@ -2400,6 +2550,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J54" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familyplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K54" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3996,6 +4151,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J97" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familyplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K97" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4482,6 +4642,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J110" t="inlineStr">
+        <ns0:is>
+          <ns0:t>barkerandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K110" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4583,6 +4748,11 @@
           <ns0:t>(361) 241-6000</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E113" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mccainplumbing@sbcglobal.net</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F113" t="inlineStr">
         <ns0:is>
           <ns0:t>9725 Leopard St</ns0:t>
@@ -4596,6 +4766,11 @@
       <ns0:c r="I113" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J113" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dwainmccainplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K113" t="inlineStr">
@@ -4640,6 +4815,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J114" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dauenhauerplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K114" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4682,6 +4862,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J115" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robinsonfamilyplumbinghvac.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K115" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -5341,6 +5526,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J132" t="inlineStr">
+        <ns0:is>
+          <ns0:t>barkerandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K132" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8496,6 +8686,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J217" t="inlineStr">
+        <ns0:is>
+          <ns0:t>irvineplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K217" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8523,6 +8718,11 @@
           <ns0:t>(657) 229-2993</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E218" t="inlineStr">
+        <ns0:is>
+          <ns0:t>leads@doitrightplumbers.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F218" t="inlineStr">
         <ns0:is>
           <ns0:t>1630 Palm St</ns0:t>
@@ -8536,6 +8736,11 @@
       <ns0:c r="I218" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J218" t="inlineStr">
+        <ns0:is>
+          <ns0:t>doitrightplumbers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K218" t="inlineStr">
@@ -8565,6 +8770,11 @@
           <ns0:t>(562) 459-6445</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E219" t="inlineStr">
+        <ns0:is>
+          <ns0:t>info@thefamilyplumber.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F219" t="inlineStr">
         <ns0:is>
           <ns0:t>3613 Briggeman Dr</ns0:t>
@@ -8578,6 +8788,11 @@
       <ns0:c r="I219" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J219" t="inlineStr">
+        <ns0:is>
+          <ns0:t>thefamilyplumber.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K219" t="inlineStr">
@@ -8696,6 +8911,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J222" t="inlineStr">
+        <ns0:is>
+          <ns0:t>allsacramento.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K222" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8738,6 +8958,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J223" t="inlineStr">
+        <ns0:is>
+          <ns0:t>stinenichols.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K223" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8780,6 +9005,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J224" t="inlineStr">
+        <ns0:is>
+          <ns0:t>miamidadeplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K224" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8881,6 +9111,11 @@
           <ns0:t>(817) 819-1471</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E227" t="inlineStr">
+        <ns0:is>
+          <ns0:t>e7d54b729aaf49ea8b2f80dae22860aa@sentry.zipify.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F227" t="inlineStr">
         <ns0:is>
           <ns0:t>Arlington, TX</ns0:t>
@@ -8894,6 +9129,11 @@
       <ns0:c r="I227" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J227" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familyfriends.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K227" t="inlineStr">
@@ -9002,6 +9242,11 @@
           <ns0:t>(813) 443-5820</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="E230" t="inlineStr">
+        <ns0:is>
+          <ns0:t>info@olinplumbinginc.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F230" t="inlineStr">
         <ns0:is>
           <ns0:t>3201 E 8th Ave</ns0:t>
@@ -9015,6 +9260,11 @@
       <ns0:c r="I230" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J230" t="inlineStr">
+        <ns0:is>
+          <ns0:t>olinplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K230" t="inlineStr">
@@ -9057,6 +9307,11 @@
       <ns0:c r="I231" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J231" t="inlineStr">
+        <ns0:is>
+          <ns0:t>barkerandsonsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K231" t="inlineStr">

</xml_diff>

<commit_message>
36% complete - 87 cities researched, 103 phones, 64 websites
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -2067,22 +2067,32 @@
       </ns0:c>
       <ns0:c r="C44" t="inlineStr">
         <ns0:is>
-          <ns0:t>Valley Plumbing</ns0:t>
+          <ns0:t>Tony's Plumbing, Heating &amp; Air</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D44" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 337-3788</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>Stockton, CA</ns0:t>
+          <ns0:t>343 E Main St Suite 420</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I44" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J44" t="inlineStr">
+        <ns0:is>
+          <ns0:t>tonysplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K44" t="inlineStr">
@@ -2574,22 +2584,32 @@
       </ns0:c>
       <ns0:c r="C55" t="inlineStr">
         <ns0:is>
-          <ns0:t>Orlando Plumbing Experts</ns0:t>
+          <ns0:t>Choice Plumbing Orlando</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D55" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(407) 422-7443</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>Orlando, FL</ns0:t>
+          <ns0:t>3550 Old Winter Garden Rd</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I55" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J55" t="inlineStr">
+        <ns0:is>
+          <ns0:t>choiceplumbingorlando.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K55" t="inlineStr">
@@ -2611,17 +2631,22 @@
       </ns0:c>
       <ns0:c r="C56" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chula Vista Plumbing</ns0:t>
+          <ns0:t>Bob the Plumber of Chula Vista</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D56" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(619) 990-7960</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chula Vista, CA</ns0:t>
+          <ns0:t>2540 Main St E</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I56" t="inlineStr">
@@ -2648,17 +2673,22 @@
       </ns0:c>
       <ns0:c r="C57" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D57" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I57" t="inlineStr">
@@ -2722,17 +2752,22 @@
       </ns0:c>
       <ns0:c r="C59" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing Pro</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D59" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F59" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G59" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I59" t="inlineStr">
@@ -2759,17 +2794,22 @@
       </ns0:c>
       <ns0:c r="C60" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston Plumbing</ns0:t>
+          <ns0:t>Transou's Plumbing &amp; Septic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D60" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 276-1263</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston-Salem, NC</ns0:t>
+          <ns0:t>101 E Devonshire St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I60" t="inlineStr">
@@ -2796,7 +2836,12 @@
       </ns0:c>
       <ns0:c r="C61" t="inlineStr">
         <ns0:is>
-          <ns0:t>Norfolk Plumbing Services</ns0:t>
+          <ns0:t>Eaton Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D61" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 913-9100</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F61" t="inlineStr">
@@ -2806,7 +2851,7 @@
       </ns0:c>
       <ns0:c r="G61" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.5+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I61" t="inlineStr">
@@ -2833,17 +2878,22 @@
       </ns0:c>
       <ns0:c r="C62" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo Plumbing Co</ns0:t>
+          <ns0:t>South Texas Plumbing Contractors</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D62" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 333-6935</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F62" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo, TX</ns0:t>
+          <ns0:t>109 Flecha Ln Suite B</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G62" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I62" t="inlineStr">
@@ -2873,6 +2923,11 @@
           <ns0:t>A-1 Plumbing</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="D63" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(806) 796-0206</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="F63" t="inlineStr">
         <ns0:is>
           <ns0:t>Lubbock, TX</ns0:t>
@@ -2880,7 +2935,7 @@
       </ns0:c>
       <ns0:c r="G63" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.5+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I63" t="inlineStr">
@@ -2907,17 +2962,22 @@
       </ns0:c>
       <ns0:c r="C64" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison Plumbing Pro</ns0:t>
+          <ns0:t>Howe Brothers Plumbing LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D64" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(608) 257-2884</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F64" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison, WI</ns0:t>
+          <ns0:t>1215 Williamson St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G64" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I64" t="inlineStr">
@@ -2944,17 +3004,22 @@
       </ns0:c>
       <ns0:c r="C65" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler Plumbing</ns0:t>
+          <ns0:t>Roy Dossey Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D65" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 963-3302</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler, AZ</ns0:t>
+          <ns0:t>120 E Highland St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.6/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I65" t="inlineStr">
@@ -2981,17 +3046,22 @@
       </ns0:c>
       <ns0:c r="C66" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving Plumbing Pro</ns0:t>
+          <ns0:t>Reeves Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D66" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 247-3763</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving, TX</ns0:t>
+          <ns0:t>13346 Bee St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I66" t="inlineStr">
@@ -3018,17 +3088,22 @@
       </ns0:c>
       <ns0:c r="C67" t="inlineStr">
         <ns0:is>
-          <ns0:t>Scottsdale Plumbing</ns0:t>
+          <ns0:t>DC Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D67" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 300-4791</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>Scottsdale, AZ</ns0:t>
+          <ns0:t>1797 W University Dr</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I67" t="inlineStr">
@@ -3055,7 +3130,12 @@
       </ns0:c>
       <ns0:c r="C68" t="inlineStr">
         <ns0:is>
-          <ns0:t>Norfolk Plumbing</ns0:t>
+          <ns0:t>Eaton Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D68" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 913-9100</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F68" t="inlineStr">
@@ -3065,7 +3145,7 @@
       </ns0:c>
       <ns0:c r="G68" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.5+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I68" t="inlineStr">
@@ -3092,17 +3172,22 @@
       </ns0:c>
       <ns0:c r="C69" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing Pro</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D69" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F69" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G69" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I69" t="inlineStr">
@@ -3166,17 +3251,22 @@
       </ns0:c>
       <ns0:c r="C71" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing Co</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D71" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I71" t="inlineStr">
@@ -3203,17 +3293,22 @@
       </ns0:c>
       <ns0:c r="C72" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston Plumbing Pro</ns0:t>
+          <ns0:t>Transou's Plumbing &amp; Septic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D72" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 276-1263</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F72" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston-Salem, NC</ns0:t>
+          <ns0:t>101 E Devonshire St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G72" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I72" t="inlineStr">
@@ -3758,17 +3853,22 @@
       </ns0:c>
       <ns0:c r="C87" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing Services</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D87" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F87" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G87" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I87" t="inlineStr">
@@ -3980,7 +4080,12 @@
       </ns0:c>
       <ns0:c r="C93" t="inlineStr">
         <ns0:is>
-          <ns0:t>Norfolk Plumbing Pro</ns0:t>
+          <ns0:t>Eaton Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D93" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 913-9100</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F93" t="inlineStr">
@@ -3990,7 +4095,7 @@
       </ns0:c>
       <ns0:c r="G93" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.5+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I93" t="inlineStr">
@@ -4703,22 +4808,32 @@
       </ns0:c>
       <ns0:c r="C112" t="inlineStr">
         <ns0:is>
-          <ns0:t>Stockton Plumbing Pro</ns0:t>
+          <ns0:t>Tony's Plumbing, Heating &amp; Air</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D112" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 337-3788</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F112" t="inlineStr">
         <ns0:is>
-          <ns0:t>Stockton, CA</ns0:t>
+          <ns0:t>343 E Main St Suite 420</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G112" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I112" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J112" t="inlineStr">
+        <ns0:is>
+          <ns0:t>tonysplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K112" t="inlineStr">
@@ -4997,17 +5112,22 @@
       </ns0:c>
       <ns0:c r="C119" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler Plumbing Pro</ns0:t>
+          <ns0:t>Roy Dossey Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D119" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 963-3302</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F119" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler, AZ</ns0:t>
+          <ns0:t>120 E Highland St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G119" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.6/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I119" t="inlineStr">
@@ -5034,17 +5154,22 @@
       </ns0:c>
       <ns0:c r="C120" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo Plumbing Services</ns0:t>
+          <ns0:t>South Texas Plumbing Contractors</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D120" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 333-6935</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F120" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo, TX</ns0:t>
+          <ns0:t>109 Flecha Ln Suite B</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G120" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I120" t="inlineStr">
@@ -5071,22 +5196,22 @@
       </ns0:c>
       <ns0:c r="C121" t="inlineStr">
         <ns0:is>
-          <ns0:t>Pelayo Plumbing</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D121" t="inlineStr">
         <ns0:is>
-          <ns0:t>214-315-7672</ns0:t>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F121" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G121" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I121" t="inlineStr">
@@ -5160,12 +5285,12 @@
       </ns0:c>
       <ns0:c r="C123" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving Plumbing Pro</ns0:t>
+          <ns0:t>Reeves Family Plumbing</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D123" t="inlineStr">
         <ns0:is>
-          <ns0:t>972-914-9804</ns0:t>
+          <ns0:t>(972) 247-3763</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="E123" t="inlineStr">
@@ -5175,12 +5300,12 @@
       </ns0:c>
       <ns0:c r="F123" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving, TX</ns0:t>
+          <ns0:t>13346 Bee St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G123" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I123" t="inlineStr">
@@ -6475,17 +6600,22 @@
       </ns0:c>
       <ns0:c r="C158" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D158" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F158" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G158" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I158" t="inlineStr">
@@ -6549,17 +6679,22 @@
       </ns0:c>
       <ns0:c r="C160" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D160" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F160" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G160" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I160" t="inlineStr">
@@ -6586,17 +6721,22 @@
       </ns0:c>
       <ns0:c r="C161" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston Plumbing</ns0:t>
+          <ns0:t>Transou's Plumbing &amp; Septic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D161" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 276-1263</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F161" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston-Salem, NC</ns0:t>
+          <ns0:t>101 E Devonshire St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G161" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I161" t="inlineStr">
@@ -7178,17 +7318,22 @@
       </ns0:c>
       <ns0:c r="C177" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D177" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F177" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G177" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I177" t="inlineStr">
@@ -7252,17 +7397,22 @@
       </ns0:c>
       <ns0:c r="C179" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D179" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F179" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G179" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I179" t="inlineStr">
@@ -7289,17 +7439,22 @@
       </ns0:c>
       <ns0:c r="C180" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston Plumbing</ns0:t>
+          <ns0:t>Transou's Plumbing &amp; Septic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D180" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 276-1263</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F180" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston-Salem, NC</ns0:t>
+          <ns0:t>101 E Devonshire St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G180" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I180" t="inlineStr">
@@ -7955,17 +8110,22 @@
       </ns0:c>
       <ns0:c r="C198" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D198" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F198" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G198" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I198" t="inlineStr">
@@ -8029,17 +8189,22 @@
       </ns0:c>
       <ns0:c r="C200" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D200" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F200" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G200" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I200" t="inlineStr">
@@ -8066,17 +8231,22 @@
       </ns0:c>
       <ns0:c r="C201" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston Plumbing</ns0:t>
+          <ns0:t>Transou's Plumbing &amp; Septic</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D201" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 276-1263</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F201" t="inlineStr">
         <ns0:is>
-          <ns0:t>Winston-Salem, NC</ns0:t>
+          <ns0:t>101 E Devonshire St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G201" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I201" t="inlineStr">
@@ -8436,17 +8606,22 @@
       </ns0:c>
       <ns0:c r="C211" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison Plumbing</ns0:t>
+          <ns0:t>Howe Brothers Plumbing LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D211" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(608) 257-2884</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F211" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison, WI</ns0:t>
+          <ns0:t>1215 Williamson St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G211" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I211" t="inlineStr">
@@ -8473,17 +8648,22 @@
       </ns0:c>
       <ns0:c r="C212" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler Plumbing</ns0:t>
+          <ns0:t>Roy Dossey Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D212" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 963-3302</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F212" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chandler, AZ</ns0:t>
+          <ns0:t>120 E Highland St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G212" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.6/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I212" t="inlineStr">
@@ -8510,17 +8690,22 @@
       </ns0:c>
       <ns0:c r="C213" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving Plumbing</ns0:t>
+          <ns0:t>Reeves Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D213" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 247-3763</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F213" t="inlineStr">
         <ns0:is>
-          <ns0:t>Irving, TX</ns0:t>
+          <ns0:t>13346 Bee St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G213" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I213" t="inlineStr">
@@ -8547,22 +8732,22 @@
       </ns0:c>
       <ns0:c r="C214" t="inlineStr">
         <ns0:is>
-          <ns0:t>Scottsdale Plumbing</ns0:t>
+          <ns0:t>DC Family Plumbing</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D214" t="inlineStr">
         <ns0:is>
-          <ns0:t>480-908-2275</ns0:t>
+          <ns0:t>(480) 300-4791</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F214" t="inlineStr">
         <ns0:is>
-          <ns0:t>Scottsdale, AZ</ns0:t>
+          <ns0:t>1797 W University Dr</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G214" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I214" t="inlineStr">
@@ -9370,17 +9555,22 @@
       </ns0:c>
       <ns0:c r="C233" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chula Vista Plumbing</ns0:t>
+          <ns0:t>Bob the Plumber of Chula Vista</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D233" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(619) 990-7960</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F233" t="inlineStr">
         <ns0:is>
-          <ns0:t>Chula Vista, CA</ns0:t>
+          <ns0:t>2540 Main St E</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G233" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I233" t="inlineStr">
@@ -9444,17 +9634,22 @@
       </ns0:c>
       <ns0:c r="C235" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland Plumbing TX</ns0:t>
+          <ns0:t>Family Ties Plumbing &amp; Construction</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D235" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(972) 824-8833</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F235" t="inlineStr">
         <ns0:is>
-          <ns0:t>Garland, TX</ns0:t>
+          <ns0:t>3906 Melcer Dr #301</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G235" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>5.0/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I235" t="inlineStr">
@@ -9518,17 +9713,22 @@
       </ns0:c>
       <ns0:c r="C237" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert Plumbing AZ</ns0:t>
+          <ns0:t>Travis &amp; Sons Plumbing &amp; Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D237" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(480) 568-2309</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F237" t="inlineStr">
         <ns0:is>
-          <ns0:t>Gilbert, AZ</ns0:t>
+          <ns0:t>1324 N Farrell Ct</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G237" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I237" t="inlineStr">
@@ -9555,17 +9755,22 @@
       </ns0:c>
       <ns0:c r="C238" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo Plumbing TX</ns0:t>
+          <ns0:t>South Texas Plumbing Contractors</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D238" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 333-6935</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F238" t="inlineStr">
         <ns0:is>
-          <ns0:t>Laredo, TX</ns0:t>
+          <ns0:t>109 Flecha Ln Suite B</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G238" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.7/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I238" t="inlineStr">
@@ -9629,17 +9834,22 @@
       </ns0:c>
       <ns0:c r="C240" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison Plumbing WI</ns0:t>
+          <ns0:t>Howe Brothers Plumbing LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D240" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(608) 257-2884</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F240" t="inlineStr">
         <ns0:is>
-          <ns0:t>Madison, WI</ns0:t>
+          <ns0:t>1215 Williamson St</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G240" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6+/5</ns0:t>
+          <ns0:t>4.9/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I240" t="inlineStr">

</xml_diff>

<commit_message>
131 phones, 88 websites, 93 cities researched
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -128,7 +128,7 @@
       </ns0:c>
       <ns0:c r="G2" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7/5 (Angi)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I2" t="inlineStr">
@@ -170,7 +170,7 @@
       </ns0:c>
       <ns0:c r="F3" t="inlineStr">
         <ns0:is>
-          <ns0:t>2361 Barton Ln, Montrose, CA 91020</ns0:t>
+          <ns0:t>2361 Barton Lane, Montrose, CA 91020</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G3" t="inlineStr">
@@ -217,12 +217,12 @@
       </ns0:c>
       <ns0:c r="F4" t="inlineStr">
         <ns0:is>
-          <ns0:t>51 Eisenhower Ln S, Lombard, IL 60148</ns0:t>
+          <ns0:t>West Chicago, IL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G4" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.8/5 (1000+ reviews)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I4" t="inlineStr">
@@ -264,12 +264,12 @@
       </ns0:c>
       <ns0:c r="F5" t="inlineStr">
         <ns0:is>
-          <ns0:t>10814 Woodedge Dr, Houston, TX 77070</ns0:t>
+          <ns0:t>Houston, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G5" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.9/5 (Best Pick)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I5" t="inlineStr">
@@ -311,12 +311,12 @@
       </ns0:c>
       <ns0:c r="F6" t="inlineStr">
         <ns0:is>
-          <ns0:t>1497 E Baseline Rd STE 110, Gilbert, AZ 85233</ns0:t>
+          <ns0:t>1497 E Baseline Rd, Gilbert, AZ 85233</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G6" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.9/5 (1,547 reviews)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I6" t="inlineStr">
@@ -358,12 +358,12 @@
       </ns0:c>
       <ns0:c r="F7" t="inlineStr">
         <ns0:is>
-          <ns0:t>8015 Castor Ave, Philadelphia, PA 19152</ns0:t>
+          <ns0:t>Philadelphia &amp; Feasterville-Trevose, PA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G7" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I7" t="inlineStr">
@@ -405,12 +405,12 @@
       </ns0:c>
       <ns0:c r="F8" t="inlineStr">
         <ns0:is>
-          <ns0:t>1875 E Borgfeld Dr, San Antonio, TX 78260</ns0:t>
+          <ns0:t>San Antonio, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G8" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>5.0/5 (1,400+ reviews)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I8" t="inlineStr">
@@ -457,12 +457,12 @@
       </ns0:c>
       <ns0:c r="F9" t="inlineStr">
         <ns0:is>
-          <ns0:t>422 21st St, San Diego, CA 92102</ns0:t>
+          <ns0:t>San Diego, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G9" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>5.0/5 (40+ years)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I9" t="inlineStr">
@@ -504,12 +504,12 @@
       </ns0:c>
       <ns0:c r="F10" t="inlineStr">
         <ns0:is>
-          <ns0:t>2615 Big Town Blvd, Mesquite, TX 75150</ns0:t>
+          <ns0:t>Dallas/DFW, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G10" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.9/5 (24,000+ reviews)</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I10" t="inlineStr">
@@ -551,12 +551,12 @@
       </ns0:c>
       <ns0:c r="F11" t="inlineStr">
         <ns0:is>
-          <ns0:t>19970 McKean Rd Bldg C, San Jose, CA 95120</ns0:t>
+          <ns0:t>San Jose, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G11" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.4/5</ns0:t>
+          <ns0:t>4.8/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I11" t="inlineStr">
@@ -598,12 +598,12 @@
       </ns0:c>
       <ns0:c r="F12" t="inlineStr">
         <ns0:is>
-          <ns0:t>2210 Melissa Oaks Ln, Austin, TX 78744</ns0:t>
+          <ns0:t>Austin, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G12" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.8/5+</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I12" t="inlineStr">
@@ -645,12 +645,12 @@
       </ns0:c>
       <ns0:c r="F13" t="inlineStr">
         <ns0:is>
-          <ns0:t>5000 W 29th Ave, Denver, CO 80212</ns0:t>
+          <ns0:t>Denver/Boulder, CO</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G13" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I13" t="inlineStr">
@@ -692,7 +692,7 @@
       </ns0:c>
       <ns0:c r="G14" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I14" t="inlineStr">
@@ -744,7 +744,7 @@
       </ns0:c>
       <ns0:c r="G15" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I15" t="inlineStr">
@@ -786,12 +786,12 @@
       </ns0:c>
       <ns0:c r="F16" t="inlineStr">
         <ns0:is>
-          <ns0:t>12009 NE Marx St</ns0:t>
+          <ns0:t>Portland, OR</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G16" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I16" t="inlineStr">
@@ -838,12 +838,12 @@
       </ns0:c>
       <ns0:c r="F17" t="inlineStr">
         <ns0:is>
-          <ns0:t>3744 Annex Ave</ns0:t>
+          <ns0:t>Nashville, TN</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G17" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.8+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I17" t="inlineStr">
@@ -885,12 +885,12 @@
       </ns0:c>
       <ns0:c r="F18" t="inlineStr">
         <ns0:is>
-          <ns0:t>900 Remount Rd</ns0:t>
+          <ns0:t>Charlotte, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G18" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I18" t="inlineStr">
@@ -932,12 +932,12 @@
       </ns0:c>
       <ns0:c r="F19" t="inlineStr">
         <ns0:is>
-          <ns0:t>9417 SW 77th Ct</ns0:t>
+          <ns0:t>Miami, FL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G19" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I19" t="inlineStr">
@@ -979,12 +979,12 @@
       </ns0:c>
       <ns0:c r="F20" t="inlineStr">
         <ns0:is>
-          <ns0:t>4381 Campbellton Rd SW</ns0:t>
+          <ns0:t>Atlanta, GA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G20" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.8+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I20" t="inlineStr">
@@ -1026,12 +1026,12 @@
       </ns0:c>
       <ns0:c r="F21" t="inlineStr">
         <ns0:is>
-          <ns0:t>5177 Fishwick Dr</ns0:t>
+          <ns0:t>Cincinnati, OH</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G21" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I21" t="inlineStr">
@@ -1073,12 +1073,12 @@
       </ns0:c>
       <ns0:c r="F22" t="inlineStr">
         <ns0:is>
-          <ns0:t>318 East 16th Avenue</ns0:t>
+          <ns0:t>Kansas City, MO</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G22" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I22" t="inlineStr">
@@ -1236,17 +1236,17 @@
       </ns0:c>
       <ns0:c r="D26" t="inlineStr">
         <ns0:is>
-          <ns0:t>(559) 445-9999</ns0:t>
+          <ns0:t>(505) 803-3170</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F26" t="inlineStr">
         <ns0:is>
-          <ns0:t>5639 W Barstow Ave</ns0:t>
+          <ns0:t>Albuquerque, NM</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G26" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I26" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </ns0:c>
       <ns0:c r="J26" t="inlineStr">
         <ns0:is>
-          <ns0:t>allstarplumbingfresno.com</ns0:t>
+          <ns0:t>familyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K26" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </ns0:c>
       <ns0:c r="F27" t="inlineStr">
         <ns0:is>
-          <ns0:t>1665 E 18th St #117</ns0:t>
+          <ns0:t>Tucson, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G27" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I27" t="inlineStr">
@@ -1345,12 +1345,12 @@
       </ns0:c>
       <ns0:c r="F28" t="inlineStr">
         <ns0:is>
-          <ns0:t>3613 Briggeman Dr</ns0:t>
+          <ns0:t>Long Beach, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G28" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I28" t="inlineStr">
@@ -1392,12 +1392,12 @@
       </ns0:c>
       <ns0:c r="F29" t="inlineStr">
         <ns0:is>
-          <ns0:t>2551 Albatross Wy</ns0:t>
+          <ns0:t>Sacramento, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G29" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I29" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </ns0:c>
       <ns0:c r="F30" t="inlineStr">
         <ns0:is>
-          <ns0:t>235 New Bern Pl #301</ns0:t>
+          <ns0:t>Raleigh, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G30" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I30" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </ns0:c>
       <ns0:c r="F31" t="inlineStr">
         <ns0:is>
-          <ns0:t>3201 E 8th Ave</ns0:t>
+          <ns0:t>Tampa, FL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G31" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.8+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I31" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </ns0:c>
       <ns0:c r="F32" t="inlineStr">
         <ns0:is>
-          <ns0:t>6843 Summer Ave, Memphis, TN 38134</ns0:t>
+          <ns0:t>Memphis, TN</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G32" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.8+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I32" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </ns0:c>
       <ns0:c r="G33" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I33" t="inlineStr">
@@ -1632,12 +1632,12 @@
       </ns0:c>
       <ns0:c r="F34" t="inlineStr">
         <ns0:is>
-          <ns0:t>10909 Show Pony Pl</ns0:t>
+          <ns0:t>Baltimore, MD</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G34" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I34" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </ns0:c>
       <ns0:c r="G35" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I35" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </ns0:c>
       <ns0:c r="D36" t="inlineStr">
         <ns0:is>
-          <ns0:t>(559) 445-9999</ns0:t>
+          <ns0:t>(505) 803-3170</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F36" t="inlineStr">
         <ns0:is>
-          <ns0:t>5639 W Barstow Ave</ns0:t>
+          <ns0:t>Albuquerque, NM</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G36" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I36" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </ns0:c>
       <ns0:c r="J36" t="inlineStr">
         <ns0:is>
-          <ns0:t>allstarplumbingfresno.com</ns0:t>
+          <ns0:t>familyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K36" t="inlineStr">
@@ -1778,12 +1778,12 @@
       </ns0:c>
       <ns0:c r="F37" t="inlineStr">
         <ns0:is>
-          <ns0:t>1665 E 18th St #117</ns0:t>
+          <ns0:t>Tucson, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G37" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I37" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </ns0:c>
       <ns0:c r="G39" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I39" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </ns0:c>
       <ns0:c r="G40" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I40" t="inlineStr">
@@ -1961,12 +1961,12 @@
       </ns0:c>
       <ns0:c r="F41" t="inlineStr">
         <ns0:is>
-          <ns0:t>152 Friedrichs Rd</ns0:t>
+          <ns0:t>New Orleans, LA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G41" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I41" t="inlineStr">
@@ -2077,12 +2077,12 @@
       </ns0:c>
       <ns0:c r="F44" t="inlineStr">
         <ns0:is>
-          <ns0:t>343 E Main St Suite 420</ns0:t>
+          <ns0:t>Stockton, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G44" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I44" t="inlineStr">
@@ -2129,12 +2129,12 @@
       </ns0:c>
       <ns0:c r="F45" t="inlineStr">
         <ns0:is>
-          <ns0:t>5705 Dale Ave</ns0:t>
+          <ns0:t>Saint Louis, MO</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G45" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I45" t="inlineStr">
@@ -2176,12 +2176,12 @@
       </ns0:c>
       <ns0:c r="F46" t="inlineStr">
         <ns0:is>
-          <ns0:t>10218 Indiana Ave</ns0:t>
+          <ns0:t>Riverside, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G46" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I46" t="inlineStr">
@@ -2223,12 +2223,12 @@
       </ns0:c>
       <ns0:c r="F47" t="inlineStr">
         <ns0:is>
-          <ns0:t>9725 Leopard St</ns0:t>
+          <ns0:t>Corpus Christi, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G47" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I47" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </ns0:c>
       <ns0:c r="F48" t="inlineStr">
         <ns0:is>
-          <ns0:t>426 Chair Ave</ns0:t>
+          <ns0:t>Lexington, KY</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G48" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I48" t="inlineStr">
@@ -2317,12 +2317,12 @@
       </ns0:c>
       <ns0:c r="F49" t="inlineStr">
         <ns0:is>
-          <ns0:t>691 Chablis Dr</ns0:t>
+          <ns0:t>Henderson, NV</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G49" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I49" t="inlineStr">
@@ -2364,12 +2364,12 @@
       </ns0:c>
       <ns0:c r="F50" t="inlineStr">
         <ns0:is>
-          <ns0:t>3900 E Miraloma Ave</ns0:t>
+          <ns0:t>Anaheim, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G50" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I50" t="inlineStr">
@@ -2411,12 +2411,12 @@
       </ns0:c>
       <ns0:c r="F51" t="inlineStr">
         <ns0:is>
-          <ns0:t>6120 A St</ns0:t>
+          <ns0:t>Anchorage, AK</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G51" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.1/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I51" t="inlineStr">
@@ -2463,12 +2463,12 @@
       </ns0:c>
       <ns0:c r="F52" t="inlineStr">
         <ns0:is>
-          <ns0:t>1630 Palm St</ns0:t>
+          <ns0:t>Santa Ana, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G52" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I52" t="inlineStr">
@@ -2547,12 +2547,12 @@
       </ns0:c>
       <ns0:c r="F54" t="inlineStr">
         <ns0:is>
-          <ns0:t>510 Newport Blvd # A109</ns0:t>
+          <ns0:t>Irvine, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G54" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I54" t="inlineStr">
@@ -2594,12 +2594,12 @@
       </ns0:c>
       <ns0:c r="F55" t="inlineStr">
         <ns0:is>
-          <ns0:t>3550 Old Winter Garden Rd</ns0:t>
+          <ns0:t>Orlando, FL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G55" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I55" t="inlineStr">
@@ -2641,12 +2641,12 @@
       </ns0:c>
       <ns0:c r="F56" t="inlineStr">
         <ns0:is>
-          <ns0:t>2540 Main St E</ns0:t>
+          <ns0:t>Chula Vista, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G56" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I56" t="inlineStr">
@@ -2683,12 +2683,12 @@
       </ns0:c>
       <ns0:c r="F57" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G57" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I57" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </ns0:c>
       <ns0:c r="F59" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G59" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I59" t="inlineStr">
@@ -2804,12 +2804,12 @@
       </ns0:c>
       <ns0:c r="F60" t="inlineStr">
         <ns0:is>
-          <ns0:t>101 E Devonshire St</ns0:t>
+          <ns0:t>Winston-Salem, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G60" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I60" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </ns0:c>
       <ns0:c r="G61" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I61" t="inlineStr">
@@ -2888,12 +2888,12 @@
       </ns0:c>
       <ns0:c r="F62" t="inlineStr">
         <ns0:is>
-          <ns0:t>109 Flecha Ln Suite B</ns0:t>
+          <ns0:t>Laredo, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G62" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I62" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </ns0:c>
       <ns0:c r="G63" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I63" t="inlineStr">
@@ -2972,12 +2972,12 @@
       </ns0:c>
       <ns0:c r="F64" t="inlineStr">
         <ns0:is>
-          <ns0:t>1215 Williamson St</ns0:t>
+          <ns0:t>Madison, WI</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G64" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I64" t="inlineStr">
@@ -3014,12 +3014,12 @@
       </ns0:c>
       <ns0:c r="F65" t="inlineStr">
         <ns0:is>
-          <ns0:t>120 E Highland St</ns0:t>
+          <ns0:t>Chandler, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G65" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I65" t="inlineStr">
@@ -3056,12 +3056,12 @@
       </ns0:c>
       <ns0:c r="F66" t="inlineStr">
         <ns0:is>
-          <ns0:t>13346 Bee St</ns0:t>
+          <ns0:t>Irving, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G66" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I66" t="inlineStr">
@@ -3098,12 +3098,12 @@
       </ns0:c>
       <ns0:c r="F67" t="inlineStr">
         <ns0:is>
-          <ns0:t>1797 W University Dr</ns0:t>
+          <ns0:t>Scottsdale, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G67" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I67" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </ns0:c>
       <ns0:c r="G68" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I68" t="inlineStr">
@@ -3182,12 +3182,12 @@
       </ns0:c>
       <ns0:c r="F69" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G69" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I69" t="inlineStr">
@@ -3261,12 +3261,12 @@
       </ns0:c>
       <ns0:c r="F71" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G71" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I71" t="inlineStr">
@@ -3303,12 +3303,12 @@
       </ns0:c>
       <ns0:c r="F72" t="inlineStr">
         <ns0:is>
-          <ns0:t>101 E Devonshire St</ns0:t>
+          <ns0:t>Winston-Salem, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G72" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I72" t="inlineStr">
@@ -3335,7 +3335,12 @@
       </ns0:c>
       <ns0:c r="C73" t="inlineStr">
         <ns0:is>
-          <ns0:t>Hialeah Plumbing</ns0:t>
+          <ns0:t>Hernandez Plumbing Co.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D73" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(305) 428-3782</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F73" t="inlineStr">
@@ -3372,7 +3377,12 @@
       </ns0:c>
       <ns0:c r="C74" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D74" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F74" t="inlineStr">
@@ -3388,6 +3398,11 @@
       <ns0:c r="I74" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J74" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K74" t="inlineStr">
@@ -3409,7 +3424,12 @@
       </ns0:c>
       <ns0:c r="C75" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D75" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F75" t="inlineStr">
@@ -3425,6 +3445,11 @@
       <ns0:c r="I75" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J75" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K75" t="inlineStr">
@@ -3446,7 +3471,12 @@
       </ns0:c>
       <ns0:c r="C76" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D76" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F76" t="inlineStr">
@@ -3462,6 +3492,11 @@
       <ns0:c r="I76" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J76" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K76" t="inlineStr">
@@ -3483,7 +3518,12 @@
       </ns0:c>
       <ns0:c r="C77" t="inlineStr">
         <ns0:is>
-          <ns0:t>Brownsville Plumbing</ns0:t>
+          <ns0:t>Robert's Repair Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D77" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 203-9993</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F77" t="inlineStr">
@@ -3499,6 +3539,11 @@
       <ns0:c r="I77" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J77" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robertsrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K77" t="inlineStr">
@@ -3863,12 +3908,12 @@
       </ns0:c>
       <ns0:c r="F87" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G87" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I87" t="inlineStr">
@@ -3932,7 +3977,12 @@
       </ns0:c>
       <ns0:c r="C89" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing Services</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D89" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F89" t="inlineStr">
@@ -3948,6 +3998,11 @@
       <ns0:c r="I89" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J89" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K89" t="inlineStr">
@@ -3969,7 +4024,12 @@
       </ns0:c>
       <ns0:c r="C90" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing Services</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D90" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F90" t="inlineStr">
@@ -3985,6 +4045,11 @@
       <ns0:c r="I90" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J90" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K90" t="inlineStr">
@@ -4095,7 +4160,7 @@
       </ns0:c>
       <ns0:c r="G93" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I93" t="inlineStr">
@@ -4243,12 +4308,12 @@
       </ns0:c>
       <ns0:c r="F97" t="inlineStr">
         <ns0:is>
-          <ns0:t>510 Newport Blvd # A109</ns0:t>
+          <ns0:t>Irvine, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G97" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I97" t="inlineStr">
@@ -4391,7 +4456,12 @@
       </ns0:c>
       <ns0:c r="C101" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing Pro</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D101" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F101" t="inlineStr">
@@ -4407,6 +4477,11 @@
       <ns0:c r="I101" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J101" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K101" t="inlineStr">
@@ -4428,7 +4503,12 @@
       </ns0:c>
       <ns0:c r="C102" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing Pro</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D102" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F102" t="inlineStr">
@@ -4444,6 +4524,11 @@
       <ns0:c r="I102" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J102" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K102" t="inlineStr">
@@ -4502,7 +4587,12 @@
       </ns0:c>
       <ns0:c r="C104" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing Pro</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D104" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F104" t="inlineStr">
@@ -4518,6 +4608,11 @@
       <ns0:c r="I104" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J104" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K104" t="inlineStr">
@@ -4734,12 +4829,12 @@
       </ns0:c>
       <ns0:c r="F110" t="inlineStr">
         <ns0:is>
-          <ns0:t>3900 E Miraloma Ave</ns0:t>
+          <ns0:t>Anaheim, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G110" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I110" t="inlineStr">
@@ -4818,12 +4913,12 @@
       </ns0:c>
       <ns0:c r="F112" t="inlineStr">
         <ns0:is>
-          <ns0:t>343 E Main St Suite 420</ns0:t>
+          <ns0:t>Stockton, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G112" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I112" t="inlineStr">
@@ -4870,12 +4965,12 @@
       </ns0:c>
       <ns0:c r="F113" t="inlineStr">
         <ns0:is>
-          <ns0:t>9725 Leopard St</ns0:t>
+          <ns0:t>Corpus Christi, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G113" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.5+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I113" t="inlineStr">
@@ -4917,12 +5012,12 @@
       </ns0:c>
       <ns0:c r="F114" t="inlineStr">
         <ns0:is>
-          <ns0:t>426 Chair Ave</ns0:t>
+          <ns0:t>Lexington, KY</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G114" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I114" t="inlineStr">
@@ -4964,12 +5059,12 @@
       </ns0:c>
       <ns0:c r="F115" t="inlineStr">
         <ns0:is>
-          <ns0:t>691 Chablis Dr</ns0:t>
+          <ns0:t>Henderson, NV</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G115" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I115" t="inlineStr">
@@ -5122,12 +5217,12 @@
       </ns0:c>
       <ns0:c r="F119" t="inlineStr">
         <ns0:is>
-          <ns0:t>120 E Highland St</ns0:t>
+          <ns0:t>Chandler, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G119" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I119" t="inlineStr">
@@ -5164,12 +5259,12 @@
       </ns0:c>
       <ns0:c r="F120" t="inlineStr">
         <ns0:is>
-          <ns0:t>109 Flecha Ln Suite B</ns0:t>
+          <ns0:t>Laredo, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G120" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I120" t="inlineStr">
@@ -5206,12 +5301,12 @@
       </ns0:c>
       <ns0:c r="F121" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G121" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I121" t="inlineStr">
@@ -5253,7 +5348,7 @@
       </ns0:c>
       <ns0:c r="G122" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.8+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I122" t="inlineStr">
@@ -5300,12 +5395,12 @@
       </ns0:c>
       <ns0:c r="F123" t="inlineStr">
         <ns0:is>
-          <ns0:t>13346 Bee St</ns0:t>
+          <ns0:t>Irving, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G123" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I123" t="inlineStr">
@@ -5638,12 +5733,12 @@
       </ns0:c>
       <ns0:c r="F132" t="inlineStr">
         <ns0:is>
-          <ns0:t>3900 E Miraloma Ave</ns0:t>
+          <ns0:t>Anaheim, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G132" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I132" t="inlineStr">
@@ -5971,7 +6066,12 @@
       </ns0:c>
       <ns0:c r="C141" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing Pro</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D141" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F141" t="inlineStr">
@@ -5987,6 +6087,11 @@
       <ns0:c r="I141" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J141" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K141" t="inlineStr">
@@ -6008,7 +6113,12 @@
       </ns0:c>
       <ns0:c r="C142" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing Pro</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D142" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F142" t="inlineStr">
@@ -6024,6 +6134,11 @@
       <ns0:c r="I142" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J142" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K142" t="inlineStr">
@@ -6082,7 +6197,12 @@
       </ns0:c>
       <ns0:c r="C144" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D144" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F144" t="inlineStr">
@@ -6098,6 +6218,11 @@
       <ns0:c r="I144" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J144" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K144" t="inlineStr">
@@ -6610,12 +6735,12 @@
       </ns0:c>
       <ns0:c r="F158" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G158" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I158" t="inlineStr">
@@ -6689,12 +6814,12 @@
       </ns0:c>
       <ns0:c r="F160" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G160" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I160" t="inlineStr">
@@ -6731,12 +6856,12 @@
       </ns0:c>
       <ns0:c r="F161" t="inlineStr">
         <ns0:is>
-          <ns0:t>101 E Devonshire St</ns0:t>
+          <ns0:t>Winston-Salem, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G161" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I161" t="inlineStr">
@@ -6763,7 +6888,12 @@
       </ns0:c>
       <ns0:c r="C162" t="inlineStr">
         <ns0:is>
-          <ns0:t>Hialeah Plumbing</ns0:t>
+          <ns0:t>Hernandez Plumbing Co.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D162" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(305) 428-3782</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F162" t="inlineStr">
@@ -6800,7 +6930,12 @@
       </ns0:c>
       <ns0:c r="C163" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D163" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F163" t="inlineStr">
@@ -6816,6 +6951,11 @@
       <ns0:c r="I163" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J163" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K163" t="inlineStr">
@@ -6837,7 +6977,12 @@
       </ns0:c>
       <ns0:c r="C164" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D164" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F164" t="inlineStr">
@@ -6853,6 +6998,11 @@
       <ns0:c r="I164" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J164" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K164" t="inlineStr">
@@ -6874,7 +7024,12 @@
       </ns0:c>
       <ns0:c r="C165" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D165" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F165" t="inlineStr">
@@ -6890,6 +7045,11 @@
       <ns0:c r="I165" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J165" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K165" t="inlineStr">
@@ -6911,7 +7071,12 @@
       </ns0:c>
       <ns0:c r="C166" t="inlineStr">
         <ns0:is>
-          <ns0:t>Brownsville Plumbing</ns0:t>
+          <ns0:t>Robert's Repair Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D166" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 203-9993</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F166" t="inlineStr">
@@ -6927,6 +7092,11 @@
       <ns0:c r="I166" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J166" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robertsrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K166" t="inlineStr">
@@ -7328,12 +7498,12 @@
       </ns0:c>
       <ns0:c r="F177" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G177" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I177" t="inlineStr">
@@ -7407,12 +7577,12 @@
       </ns0:c>
       <ns0:c r="F179" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G179" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I179" t="inlineStr">
@@ -7449,12 +7619,12 @@
       </ns0:c>
       <ns0:c r="F180" t="inlineStr">
         <ns0:is>
-          <ns0:t>101 E Devonshire St</ns0:t>
+          <ns0:t>Winston-Salem, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G180" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I180" t="inlineStr">
@@ -7481,7 +7651,12 @@
       </ns0:c>
       <ns0:c r="C181" t="inlineStr">
         <ns0:is>
-          <ns0:t>Hialeah Plumbing</ns0:t>
+          <ns0:t>Hernandez Plumbing Co.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D181" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(305) 428-3782</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F181" t="inlineStr">
@@ -7518,7 +7693,12 @@
       </ns0:c>
       <ns0:c r="C182" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D182" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F182" t="inlineStr">
@@ -7534,6 +7714,11 @@
       <ns0:c r="I182" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J182" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K182" t="inlineStr">
@@ -7555,7 +7740,12 @@
       </ns0:c>
       <ns0:c r="C183" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D183" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F183" t="inlineStr">
@@ -7571,6 +7761,11 @@
       <ns0:c r="I183" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J183" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K183" t="inlineStr">
@@ -7592,7 +7787,12 @@
       </ns0:c>
       <ns0:c r="C184" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D184" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F184" t="inlineStr">
@@ -7608,6 +7808,11 @@
       <ns0:c r="I184" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J184" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K184" t="inlineStr">
@@ -7629,7 +7834,12 @@
       </ns0:c>
       <ns0:c r="C185" t="inlineStr">
         <ns0:is>
-          <ns0:t>Brownsville Plumbing</ns0:t>
+          <ns0:t>Robert's Repair Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D185" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 203-9993</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F185" t="inlineStr">
@@ -7645,6 +7855,11 @@
       <ns0:c r="I185" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J185" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robertsrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K185" t="inlineStr">
@@ -8120,12 +8335,12 @@
       </ns0:c>
       <ns0:c r="F198" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G198" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I198" t="inlineStr">
@@ -8199,12 +8414,12 @@
       </ns0:c>
       <ns0:c r="F200" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G200" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I200" t="inlineStr">
@@ -8241,12 +8456,12 @@
       </ns0:c>
       <ns0:c r="F201" t="inlineStr">
         <ns0:is>
-          <ns0:t>101 E Devonshire St</ns0:t>
+          <ns0:t>Winston-Salem, NC</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G201" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I201" t="inlineStr">
@@ -8273,7 +8488,12 @@
       </ns0:c>
       <ns0:c r="C202" t="inlineStr">
         <ns0:is>
-          <ns0:t>Hialeah Plumbing</ns0:t>
+          <ns0:t>Hernandez Plumbing Co.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D202" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(305) 428-3782</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F202" t="inlineStr">
@@ -8310,7 +8530,12 @@
       </ns0:c>
       <ns0:c r="C203" t="inlineStr">
         <ns0:is>
-          <ns0:t>Modesto Plumbing</ns0:t>
+          <ns0:t>Herk's Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D203" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(209) 496-1388</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F203" t="inlineStr">
@@ -8326,6 +8551,11 @@
       <ns0:c r="I203" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J203" t="inlineStr">
+        <ns0:is>
+          <ns0:t>herksplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K203" t="inlineStr">
@@ -8347,7 +8577,12 @@
       </ns0:c>
       <ns0:c r="C204" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fontana Plumbing</ns0:t>
+          <ns0:t>Family Ties Air, Plumbing, &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D204" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2558</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F204" t="inlineStr">
@@ -8363,6 +8598,11 @@
       <ns0:c r="I204" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J204" t="inlineStr">
+        <ns0:is>
+          <ns0:t>familytiesair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K204" t="inlineStr">
@@ -8384,7 +8624,12 @@
       </ns0:c>
       <ns0:c r="C205" t="inlineStr">
         <ns0:is>
-          <ns0:t>Moreno Valley Plumbing</ns0:t>
+          <ns0:t>McPherson Bros Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D205" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(833) 627-2767</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F205" t="inlineStr">
@@ -8400,6 +8645,11 @@
       <ns0:c r="I205" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J205" t="inlineStr">
+        <ns0:is>
+          <ns0:t>mcphersonbros.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K205" t="inlineStr">
@@ -8421,7 +8671,12 @@
       </ns0:c>
       <ns0:c r="C206" t="inlineStr">
         <ns0:is>
-          <ns0:t>Brownsville Plumbing</ns0:t>
+          <ns0:t>Robert's Repair Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D206" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(956) 203-9993</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F206" t="inlineStr">
@@ -8437,6 +8692,11 @@
       <ns0:c r="I206" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J206" t="inlineStr">
+        <ns0:is>
+          <ns0:t>robertsrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K206" t="inlineStr">
@@ -8616,12 +8876,12 @@
       </ns0:c>
       <ns0:c r="F211" t="inlineStr">
         <ns0:is>
-          <ns0:t>1215 Williamson St</ns0:t>
+          <ns0:t>Madison, WI</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G211" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I211" t="inlineStr">
@@ -8658,12 +8918,12 @@
       </ns0:c>
       <ns0:c r="F212" t="inlineStr">
         <ns0:is>
-          <ns0:t>120 E Highland St</ns0:t>
+          <ns0:t>Chandler, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G212" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.6/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I212" t="inlineStr">
@@ -8700,12 +8960,12 @@
       </ns0:c>
       <ns0:c r="F213" t="inlineStr">
         <ns0:is>
-          <ns0:t>13346 Bee St</ns0:t>
+          <ns0:t>Irving, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G213" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I213" t="inlineStr">
@@ -8742,12 +9002,12 @@
       </ns0:c>
       <ns0:c r="F214" t="inlineStr">
         <ns0:is>
-          <ns0:t>1797 W University Dr</ns0:t>
+          <ns0:t>Scottsdale, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G214" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.7+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I214" t="inlineStr">
@@ -8858,12 +9118,12 @@
       </ns0:c>
       <ns0:c r="F217" t="inlineStr">
         <ns0:is>
-          <ns0:t>3349 Michelson Dr</ns0:t>
+          <ns0:t>Irvine, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G217" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I217" t="inlineStr">
@@ -8910,12 +9170,12 @@
       </ns0:c>
       <ns0:c r="F218" t="inlineStr">
         <ns0:is>
-          <ns0:t>1630 Palm St</ns0:t>
+          <ns0:t>Santa Ana, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G218" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I218" t="inlineStr">
@@ -8962,12 +9222,12 @@
       </ns0:c>
       <ns0:c r="F219" t="inlineStr">
         <ns0:is>
-          <ns0:t>3613 Briggeman Dr</ns0:t>
+          <ns0:t>Long Beach, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G219" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I219" t="inlineStr">
@@ -9083,12 +9343,12 @@
       </ns0:c>
       <ns0:c r="F222" t="inlineStr">
         <ns0:is>
-          <ns0:t>1875 Diesel Dr Suite 10</ns0:t>
+          <ns0:t>Sacramento, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G222" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I222" t="inlineStr">
@@ -9130,12 +9390,12 @@
       </ns0:c>
       <ns0:c r="F223" t="inlineStr">
         <ns0:is>
-          <ns0:t>318 East 16th Avenue</ns0:t>
+          <ns0:t>Kansas City, MO</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G223" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I223" t="inlineStr">
@@ -9177,12 +9437,12 @@
       </ns0:c>
       <ns0:c r="F224" t="inlineStr">
         <ns0:is>
-          <ns0:t>9417 SW 77th Ct</ns0:t>
+          <ns0:t>Miami, FL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G224" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I224" t="inlineStr">
@@ -9308,7 +9568,7 @@
       </ns0:c>
       <ns0:c r="G227" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I227" t="inlineStr">
@@ -9350,12 +9610,12 @@
       </ns0:c>
       <ns0:c r="F228" t="inlineStr">
         <ns0:is>
-          <ns0:t>152 Friedrichs Rd</ns0:t>
+          <ns0:t>New Orleans, LA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G228" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I228" t="inlineStr">
@@ -9434,12 +9694,12 @@
       </ns0:c>
       <ns0:c r="F230" t="inlineStr">
         <ns0:is>
-          <ns0:t>3201 E 8th Ave</ns0:t>
+          <ns0:t>Tampa, FL</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G230" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I230" t="inlineStr">
@@ -9481,12 +9741,12 @@
       </ns0:c>
       <ns0:c r="F231" t="inlineStr">
         <ns0:is>
-          <ns0:t>3900 E Miraloma Ave</ns0:t>
+          <ns0:t>Anaheim, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G231" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I231" t="inlineStr">
@@ -9565,12 +9825,12 @@
       </ns0:c>
       <ns0:c r="F233" t="inlineStr">
         <ns0:is>
-          <ns0:t>2540 Main St E</ns0:t>
+          <ns0:t>Chula Vista, CA</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G233" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I233" t="inlineStr">
@@ -9644,12 +9904,12 @@
       </ns0:c>
       <ns0:c r="F235" t="inlineStr">
         <ns0:is>
-          <ns0:t>3906 Melcer Dr #301</ns0:t>
+          <ns0:t>Garland, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G235" t="inlineStr">
         <ns0:is>
-          <ns0:t>5.0/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I235" t="inlineStr">
@@ -9723,12 +9983,12 @@
       </ns0:c>
       <ns0:c r="F237" t="inlineStr">
         <ns0:is>
-          <ns0:t>1324 N Farrell Ct</ns0:t>
+          <ns0:t>Gilbert, AZ</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G237" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.8/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I237" t="inlineStr">
@@ -9765,12 +10025,12 @@
       </ns0:c>
       <ns0:c r="F238" t="inlineStr">
         <ns0:is>
-          <ns0:t>109 Flecha Ln Suite B</ns0:t>
+          <ns0:t>Laredo, TX</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G238" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.7/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I238" t="inlineStr">
@@ -9844,12 +10104,12 @@
       </ns0:c>
       <ns0:c r="F240" t="inlineStr">
         <ns0:is>
-          <ns0:t>1215 Williamson St</ns0:t>
+          <ns0:t>Madison, WI</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="G240" t="inlineStr">
         <ns0:is>
-          <ns0:t>4.9/5</ns0:t>
+          <ns0:t>4.6+/5</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="I240" t="inlineStr">

</xml_diff>

<commit_message>
159 phones, 111 websites, 99 cities researched
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -3565,7 +3565,12 @@
       </ns0:c>
       <ns0:c r="C78" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fayetteville Plumbing</ns0:t>
+          <ns0:t>Woods Plumbing Service LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D78" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(910) 920-3908</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F78" t="inlineStr">
@@ -3581,6 +3586,11 @@
       <ns0:c r="I78" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J78" t="inlineStr">
+        <ns0:is>
+          <ns0:t>woodsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K78" t="inlineStr">
@@ -3602,7 +3612,12 @@
       </ns0:c>
       <ns0:c r="C79" t="inlineStr">
         <ns0:is>
-          <ns0:t>HB Plumbing Pro</ns0:t>
+          <ns0:t>DeVinney Plumbing, Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D79" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(714) 375-0126</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F79" t="inlineStr">
@@ -3618,6 +3633,11 @@
       <ns0:c r="I79" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J79" t="inlineStr">
+        <ns0:is>
+          <ns0:t>devinneyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K79" t="inlineStr">
@@ -3676,7 +3696,12 @@
       </ns0:c>
       <ns0:c r="C81" t="inlineStr">
         <ns0:is>
-          <ns0:t>Newport News Plumbing</ns0:t>
+          <ns0:t>Blair's Plumbing Repair &amp; Drains</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D81" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 719-1236</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F81" t="inlineStr">
@@ -3692,6 +3717,11 @@
       <ns0:c r="I81" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J81" t="inlineStr">
+        <ns0:is>
+          <ns0:t>blairsplumbingrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K81" t="inlineStr">
@@ -3713,7 +3743,12 @@
       </ns0:c>
       <ns0:c r="C82" t="inlineStr">
         <ns0:is>
-          <ns0:t>Tallahassee Plumbing</ns0:t>
+          <ns0:t>White's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D82" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(850) 576-3510</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F82" t="inlineStr">
@@ -3729,6 +3764,11 @@
       <ns0:c r="I82" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J82" t="inlineStr">
+        <ns0:is>
+          <ns0:t>whitesplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K82" t="inlineStr">
@@ -3750,7 +3790,12 @@
       </ns0:c>
       <ns0:c r="C83" t="inlineStr">
         <ns0:is>
-          <ns0:t>Santa Clarita Plumbing</ns0:t>
+          <ns0:t>Matthew's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D83" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 299-6707</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F83" t="inlineStr">
@@ -3787,7 +3832,12 @@
       </ns0:c>
       <ns0:c r="C84" t="inlineStr">
         <ns0:is>
-          <ns0:t>Durham Plumbing</ns0:t>
+          <ns0:t>Brown Brothers Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D84" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(919) 220-2554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F84" t="inlineStr">
@@ -3803,6 +3853,11 @@
       <ns0:c r="I84" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J84" t="inlineStr">
+        <ns0:is>
+          <ns0:t>brownbrothers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K84" t="inlineStr">
@@ -5464,7 +5519,12 @@
       </ns0:c>
       <ns0:c r="C125" t="inlineStr">
         <ns0:is>
-          <ns0:t>Santa Clarita Plumbing</ns0:t>
+          <ns0:t>Matthew's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D125" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 299-6707</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F125" t="inlineStr">
@@ -5501,7 +5561,12 @@
       </ns0:c>
       <ns0:c r="C126" t="inlineStr">
         <ns0:is>
-          <ns0:t>Durham Plumbing Pro</ns0:t>
+          <ns0:t>Brown Brothers Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D126" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(919) 220-2554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F126" t="inlineStr">
@@ -5517,6 +5582,11 @@
       <ns0:c r="I126" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J126" t="inlineStr">
+        <ns0:is>
+          <ns0:t>brownbrothers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K126" t="inlineStr">
@@ -6355,7 +6425,12 @@
       </ns0:c>
       <ns0:c r="C148" t="inlineStr">
         <ns0:is>
-          <ns0:t>HB Plumbing Pro</ns0:t>
+          <ns0:t>DeVinney Plumbing, Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D148" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(714) 375-0126</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F148" t="inlineStr">
@@ -6371,6 +6446,11 @@
       <ns0:c r="I148" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J148" t="inlineStr">
+        <ns0:is>
+          <ns0:t>devinneyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K148" t="inlineStr">
@@ -6429,7 +6509,12 @@
       </ns0:c>
       <ns0:c r="C150" t="inlineStr">
         <ns0:is>
-          <ns0:t>Newport News Plumbing</ns0:t>
+          <ns0:t>Blair's Plumbing Repair &amp; Drains</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D150" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 719-1236</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F150" t="inlineStr">
@@ -6445,6 +6530,11 @@
       <ns0:c r="I150" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J150" t="inlineStr">
+        <ns0:is>
+          <ns0:t>blairsplumbingrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K150" t="inlineStr">
@@ -6466,7 +6556,12 @@
       </ns0:c>
       <ns0:c r="C151" t="inlineStr">
         <ns0:is>
-          <ns0:t>Tallahassee Plumbing</ns0:t>
+          <ns0:t>White's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D151" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(850) 576-3510</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F151" t="inlineStr">
@@ -6482,6 +6577,11 @@
       <ns0:c r="I151" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J151" t="inlineStr">
+        <ns0:is>
+          <ns0:t>whitesplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K151" t="inlineStr">
@@ -6503,7 +6603,12 @@
       </ns0:c>
       <ns0:c r="C152" t="inlineStr">
         <ns0:is>
-          <ns0:t>Santa Clarita Plumbing</ns0:t>
+          <ns0:t>Matthew's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D152" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 299-6707</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F152" t="inlineStr">
@@ -6540,7 +6645,12 @@
       </ns0:c>
       <ns0:c r="C153" t="inlineStr">
         <ns0:is>
-          <ns0:t>Durham Plumbing</ns0:t>
+          <ns0:t>Brown Brothers Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D153" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(919) 220-2554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F153" t="inlineStr">
@@ -6556,6 +6666,11 @@
       <ns0:c r="I153" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J153" t="inlineStr">
+        <ns0:is>
+          <ns0:t>brownbrothers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K153" t="inlineStr">
@@ -7118,7 +7233,12 @@
       </ns0:c>
       <ns0:c r="C167" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fayetteville Plumbing</ns0:t>
+          <ns0:t>Woods Plumbing Service LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D167" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(910) 920-3908</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F167" t="inlineStr">
@@ -7134,6 +7254,11 @@
       <ns0:c r="I167" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J167" t="inlineStr">
+        <ns0:is>
+          <ns0:t>woodsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K167" t="inlineStr">
@@ -7155,7 +7280,12 @@
       </ns0:c>
       <ns0:c r="C168" t="inlineStr">
         <ns0:is>
-          <ns0:t>HB Plumbing</ns0:t>
+          <ns0:t>DeVinney Plumbing, Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D168" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(714) 375-0126</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F168" t="inlineStr">
@@ -7171,6 +7301,11 @@
       <ns0:c r="I168" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J168" t="inlineStr">
+        <ns0:is>
+          <ns0:t>devinneyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K168" t="inlineStr">
@@ -7229,7 +7364,12 @@
       </ns0:c>
       <ns0:c r="C170" t="inlineStr">
         <ns0:is>
-          <ns0:t>Newport News Plumbing</ns0:t>
+          <ns0:t>Blair's Plumbing Repair &amp; Drains</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D170" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 719-1236</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F170" t="inlineStr">
@@ -7245,6 +7385,11 @@
       <ns0:c r="I170" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J170" t="inlineStr">
+        <ns0:is>
+          <ns0:t>blairsplumbingrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K170" t="inlineStr">
@@ -7266,7 +7411,12 @@
       </ns0:c>
       <ns0:c r="C171" t="inlineStr">
         <ns0:is>
-          <ns0:t>Tallahassee Plumbing</ns0:t>
+          <ns0:t>White's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D171" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(850) 576-3510</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F171" t="inlineStr">
@@ -7282,6 +7432,11 @@
       <ns0:c r="I171" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J171" t="inlineStr">
+        <ns0:is>
+          <ns0:t>whitesplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K171" t="inlineStr">
@@ -7303,7 +7458,12 @@
       </ns0:c>
       <ns0:c r="C172" t="inlineStr">
         <ns0:is>
-          <ns0:t>Santa Clarita Plumbing</ns0:t>
+          <ns0:t>Matthew's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D172" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 299-6707</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F172" t="inlineStr">
@@ -7340,7 +7500,12 @@
       </ns0:c>
       <ns0:c r="C173" t="inlineStr">
         <ns0:is>
-          <ns0:t>Durham Plumbing</ns0:t>
+          <ns0:t>Brown Brothers Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D173" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(919) 220-2554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F173" t="inlineStr">
@@ -7356,6 +7521,11 @@
       <ns0:c r="I173" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J173" t="inlineStr">
+        <ns0:is>
+          <ns0:t>brownbrothers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K173" t="inlineStr">
@@ -7881,7 +8051,12 @@
       </ns0:c>
       <ns0:c r="C186" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fayetteville Plumbing</ns0:t>
+          <ns0:t>Woods Plumbing Service LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D186" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(910) 920-3908</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F186" t="inlineStr">
@@ -7897,6 +8072,11 @@
       <ns0:c r="I186" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J186" t="inlineStr">
+        <ns0:is>
+          <ns0:t>woodsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K186" t="inlineStr">
@@ -7918,7 +8098,12 @@
       </ns0:c>
       <ns0:c r="C187" t="inlineStr">
         <ns0:is>
-          <ns0:t>HB Plumbing</ns0:t>
+          <ns0:t>DeVinney Plumbing, Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D187" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(714) 375-0126</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F187" t="inlineStr">
@@ -7934,6 +8119,11 @@
       <ns0:c r="I187" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J187" t="inlineStr">
+        <ns0:is>
+          <ns0:t>devinneyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K187" t="inlineStr">
@@ -7992,7 +8182,12 @@
       </ns0:c>
       <ns0:c r="C189" t="inlineStr">
         <ns0:is>
-          <ns0:t>Newport News Plumbing</ns0:t>
+          <ns0:t>Blair's Plumbing Repair &amp; Drains</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D189" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 719-1236</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F189" t="inlineStr">
@@ -8008,6 +8203,11 @@
       <ns0:c r="I189" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J189" t="inlineStr">
+        <ns0:is>
+          <ns0:t>blairsplumbingrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K189" t="inlineStr">
@@ -8029,7 +8229,12 @@
       </ns0:c>
       <ns0:c r="C190" t="inlineStr">
         <ns0:is>
-          <ns0:t>Tallahassee Plumbing</ns0:t>
+          <ns0:t>White's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D190" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(850) 576-3510</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F190" t="inlineStr">
@@ -8045,6 +8250,11 @@
       <ns0:c r="I190" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J190" t="inlineStr">
+        <ns0:is>
+          <ns0:t>whitesplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K190" t="inlineStr">
@@ -8066,7 +8276,12 @@
       </ns0:c>
       <ns0:c r="C191" t="inlineStr">
         <ns0:is>
-          <ns0:t>Santa Clarita Plumbing</ns0:t>
+          <ns0:t>Matthew's Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D191" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 299-6707</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F191" t="inlineStr">
@@ -8103,7 +8318,12 @@
       </ns0:c>
       <ns0:c r="C192" t="inlineStr">
         <ns0:is>
-          <ns0:t>Durham Plumbing</ns0:t>
+          <ns0:t>Brown Brothers Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D192" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(919) 220-2554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F192" t="inlineStr">
@@ -8119,6 +8339,11 @@
       <ns0:c r="I192" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J192" t="inlineStr">
+        <ns0:is>
+          <ns0:t>brownbrothers.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K192" t="inlineStr">
@@ -8718,7 +8943,12 @@
       </ns0:c>
       <ns0:c r="C207" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fayetteville Plumbing</ns0:t>
+          <ns0:t>Woods Plumbing Service LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D207" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(910) 920-3908</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F207" t="inlineStr">
@@ -8734,6 +8964,11 @@
       <ns0:c r="I207" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J207" t="inlineStr">
+        <ns0:is>
+          <ns0:t>woodsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K207" t="inlineStr">
@@ -8755,7 +8990,12 @@
       </ns0:c>
       <ns0:c r="C208" t="inlineStr">
         <ns0:is>
-          <ns0:t>HB Plumbing</ns0:t>
+          <ns0:t>DeVinney Plumbing, Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D208" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(714) 375-0126</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F208" t="inlineStr">
@@ -8771,6 +9011,11 @@
       <ns0:c r="I208" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J208" t="inlineStr">
+        <ns0:is>
+          <ns0:t>devinneyplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K208" t="inlineStr">
@@ -8829,7 +9074,12 @@
       </ns0:c>
       <ns0:c r="C210" t="inlineStr">
         <ns0:is>
-          <ns0:t>Newport News Plumbing</ns0:t>
+          <ns0:t>Blair's Plumbing Repair &amp; Drains</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D210" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(757) 719-1236</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F210" t="inlineStr">
@@ -8845,6 +9095,11 @@
       <ns0:c r="I210" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J210" t="inlineStr">
+        <ns0:is>
+          <ns0:t>blairsplumbingrepair.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K210" t="inlineStr">

</xml_diff>

<commit_message>
175 phones, 119 websites, 105 cities researched
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -3916,7 +3916,12 @@
       </ns0:c>
       <ns0:c r="C86" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D86" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F86" t="inlineStr">
@@ -3995,7 +4000,12 @@
       </ns0:c>
       <ns0:c r="C88" t="inlineStr">
         <ns0:is>
-          <ns0:t>Spokane Plumbing</ns0:t>
+          <ns0:t>Shaw Plumbing Heating &amp; Air Conditioning</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D88" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(509) 642-6166</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F88" t="inlineStr">
@@ -4011,6 +4021,11 @@
       <ns0:c r="I88" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J88" t="inlineStr">
+        <ns0:is>
+          <ns0:t>shawplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K88" t="inlineStr">
@@ -4126,7 +4141,12 @@
       </ns0:c>
       <ns0:c r="C91" t="inlineStr">
         <ns0:is>
-          <ns0:t>San Bernardino Plumbing</ns0:t>
+          <ns0:t>Thompson Family Plumbing &amp; Drain</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D91" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(909) 332-2838</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F91" t="inlineStr">
@@ -4142,6 +4162,11 @@
       <ns0:c r="I91" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J91" t="inlineStr">
+        <ns0:is>
+          <ns0:t>thompsonfamily.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K91" t="inlineStr">
@@ -4163,7 +4188,12 @@
       </ns0:c>
       <ns0:c r="C92" t="inlineStr">
         <ns0:is>
-          <ns0:t>Huntsville Plumbing</ns0:t>
+          <ns0:t>Dean Plumbing Company Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D92" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(256) 883-6130</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F92" t="inlineStr">
@@ -4179,6 +4209,11 @@
       <ns0:c r="I92" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J92" t="inlineStr">
+        <ns0:is>
+          <ns0:t>deanplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K92" t="inlineStr">
@@ -4242,7 +4277,12 @@
       </ns0:c>
       <ns0:c r="C94" t="inlineStr">
         <ns0:is>
-          <ns0:t>Baton Rouge Plumbing</ns0:t>
+          <ns0:t>Trinity Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D94" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(225) 501-5554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F94" t="inlineStr">
@@ -4279,7 +4319,12 @@
       </ns0:c>
       <ns0:c r="C95" t="inlineStr">
         <ns0:is>
-          <ns0:t>Port St. Lucie Plumbing</ns0:t>
+          <ns0:t>First Choice Plus Plumbing &amp; Air</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D95" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(772) 275-3760</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F95" t="inlineStr">
@@ -4295,6 +4340,11 @@
       <ns0:c r="I95" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J95" t="inlineStr">
+        <ns0:is>
+          <ns0:t>firstchoice.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K95" t="inlineStr">
@@ -4726,7 +4776,12 @@
       </ns0:c>
       <ns0:c r="C106" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing Pro</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D106" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F106" t="inlineStr">
@@ -5645,7 +5700,12 @@
       </ns0:c>
       <ns0:c r="C128" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing Pro</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D128" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F128" t="inlineStr">
@@ -5877,7 +5937,12 @@
       </ns0:c>
       <ns0:c r="C134" t="inlineStr">
         <ns0:is>
-          <ns0:t>Huntsville Plumbing</ns0:t>
+          <ns0:t>Dean Plumbing Company Inc.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D134" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(256) 883-6130</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F134" t="inlineStr">
@@ -5893,6 +5958,11 @@
       <ns0:c r="I134" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J134" t="inlineStr">
+        <ns0:is>
+          <ns0:t>deanplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K134" t="inlineStr">
@@ -5914,7 +5984,12 @@
       </ns0:c>
       <ns0:c r="C135" t="inlineStr">
         <ns0:is>
-          <ns0:t>Baton Rouge Plumbing</ns0:t>
+          <ns0:t>Trinity Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D135" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(225) 501-5554</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F135" t="inlineStr">
@@ -6729,7 +6804,12 @@
       </ns0:c>
       <ns0:c r="C155" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D155" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F155" t="inlineStr">
@@ -6766,7 +6846,12 @@
       </ns0:c>
       <ns0:c r="C156" t="inlineStr">
         <ns0:is>
-          <ns0:t>Spokane Plumbing</ns0:t>
+          <ns0:t>Shaw Plumbing Heating &amp; Air Conditioning</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D156" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(509) 642-6166</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F156" t="inlineStr">
@@ -6782,6 +6867,11 @@
       <ns0:c r="I156" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J156" t="inlineStr">
+        <ns0:is>
+          <ns0:t>shawplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K156" t="inlineStr">
@@ -7584,7 +7674,12 @@
       </ns0:c>
       <ns0:c r="C175" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D175" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F175" t="inlineStr">
@@ -7621,7 +7716,12 @@
       </ns0:c>
       <ns0:c r="C176" t="inlineStr">
         <ns0:is>
-          <ns0:t>Spokane Plumbing</ns0:t>
+          <ns0:t>Shaw Plumbing Heating &amp; Air Conditioning</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D176" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(509) 642-6166</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F176" t="inlineStr">
@@ -7637,6 +7737,11 @@
       <ns0:c r="I176" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J176" t="inlineStr">
+        <ns0:is>
+          <ns0:t>shawplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K176" t="inlineStr">
@@ -8402,7 +8507,12 @@
       </ns0:c>
       <ns0:c r="C194" t="inlineStr">
         <ns0:is>
-          <ns0:t>Shreveport Plumbing</ns0:t>
+          <ns0:t>Bobby L. Greene Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D194" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(318) 929-6574</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F194" t="inlineStr">
@@ -8439,7 +8549,12 @@
       </ns0:c>
       <ns0:c r="C195" t="inlineStr">
         <ns0:is>
-          <ns0:t>Spokane Plumbing</ns0:t>
+          <ns0:t>Shaw Plumbing Heating &amp; Air Conditioning</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D195" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(509) 642-6166</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F195" t="inlineStr">
@@ -8455,6 +8570,11 @@
       <ns0:c r="I195" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J195" t="inlineStr">
+        <ns0:is>
+          <ns0:t>shawplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K195" t="inlineStr">

</xml_diff>

<commit_message>
190 phones, 125 websites, 112 cities researched
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -4366,7 +4366,12 @@
       </ns0:c>
       <ns0:c r="C96" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oceanside Plumbing</ns0:t>
+          <ns0:t>Parmley Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D96" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(858) 229-3341</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F96" t="inlineStr">
@@ -4450,7 +4455,12 @@
       </ns0:c>
       <ns0:c r="C98" t="inlineStr">
         <ns0:is>
-          <ns0:t>Jersey City Plumbing</ns0:t>
+          <ns0:t>Carmine P. Aumenta &amp; Sons Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D98" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(201) 451-8008</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F98" t="inlineStr">
@@ -4487,7 +4497,12 @@
       </ns0:c>
       <ns0:c r="C99" t="inlineStr">
         <ns0:is>
-          <ns0:t>Aurora Plumbing</ns0:t>
+          <ns0:t>Aurora Plumbing Company</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D99" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(303) 366-5828</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F99" t="inlineStr">
@@ -4503,6 +4518,11 @@
       <ns0:c r="I99" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J99" t="inlineStr">
+        <ns0:is>
+          <ns0:t>auroraplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K99" t="inlineStr">
@@ -4524,7 +4544,12 @@
       </ns0:c>
       <ns0:c r="C100" t="inlineStr">
         <ns0:is>
-          <ns0:t>Akron Plumbing Pro</ns0:t>
+          <ns0:t>J&amp;J Plumbing, Heating, Cooling, &amp; Electric</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D100" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(330) 967-0147</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F100" t="inlineStr">
@@ -4540,6 +4565,11 @@
       <ns0:c r="I100" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J100" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jandjplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K100" t="inlineStr">
@@ -4655,7 +4685,12 @@
       </ns0:c>
       <ns0:c r="C103" t="inlineStr">
         <ns0:is>
-          <ns0:t>Glendale CA Plumbing</ns0:t>
+          <ns0:t>Morrissey Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D103" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(818) 915-6630</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F103" t="inlineStr">
@@ -4671,6 +4706,11 @@
       <ns0:c r="I103" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J103" t="inlineStr">
+        <ns0:is>
+          <ns0:t>morrisseyfamily.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K103" t="inlineStr">
@@ -4739,7 +4779,12 @@
       </ns0:c>
       <ns0:c r="C105" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oxnard Plumbing</ns0:t>
+          <ns0:t>Salinas and Sons Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D105" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(805) 486-7030</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F105" t="inlineStr">
@@ -4818,7 +4863,12 @@
       </ns0:c>
       <ns0:c r="C107" t="inlineStr">
         <ns0:is>
-          <ns0:t>Yonkers Plumbing</ns0:t>
+          <ns0:t>JP Plumbing and Sewer</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D107" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(914) 527-2773</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F107" t="inlineStr">
@@ -5742,7 +5792,12 @@
       </ns0:c>
       <ns0:c r="C129" t="inlineStr">
         <ns0:is>
-          <ns0:t>Yonkers Plumbing Pro</ns0:t>
+          <ns0:t>JP Plumbing and Sewer</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D129" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(914) 527-2773</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F129" t="inlineStr">
@@ -6063,7 +6118,12 @@
       </ns0:c>
       <ns0:c r="C137" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oceanside Plumbing</ns0:t>
+          <ns0:t>Parmley Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D137" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(858) 229-3341</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F137" t="inlineStr">
@@ -6100,7 +6160,12 @@
       </ns0:c>
       <ns0:c r="C138" t="inlineStr">
         <ns0:is>
-          <ns0:t>Jersey City Plumbing</ns0:t>
+          <ns0:t>Carmine P. Aumenta &amp; Sons Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D138" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(201) 451-8008</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F138" t="inlineStr">
@@ -6137,7 +6202,12 @@
       </ns0:c>
       <ns0:c r="C139" t="inlineStr">
         <ns0:is>
-          <ns0:t>Aurora Plumbing CO</ns0:t>
+          <ns0:t>Aurora Plumbing Company</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D139" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(303) 366-5828</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F139" t="inlineStr">
@@ -6153,6 +6223,11 @@
       <ns0:c r="I139" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J139" t="inlineStr">
+        <ns0:is>
+          <ns0:t>auroraplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K139" t="inlineStr">
@@ -6174,7 +6249,12 @@
       </ns0:c>
       <ns0:c r="C140" t="inlineStr">
         <ns0:is>
-          <ns0:t>Akron Plumbing Pro</ns0:t>
+          <ns0:t>J&amp;J Plumbing, Heating, Cooling, &amp; Electric</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D140" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(330) 967-0147</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F140" t="inlineStr">
@@ -6190,6 +6270,11 @@
       <ns0:c r="I140" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J140" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jandjplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K140" t="inlineStr">
@@ -6305,7 +6390,12 @@
       </ns0:c>
       <ns0:c r="C143" t="inlineStr">
         <ns0:is>
-          <ns0:t>Glendale CA Plumbing</ns0:t>
+          <ns0:t>Morrissey Family Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D143" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(818) 915-6630</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F143" t="inlineStr">
@@ -6321,6 +6411,11 @@
       <ns0:c r="I143" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J143" t="inlineStr">
+        <ns0:is>
+          <ns0:t>morrisseyfamily.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K143" t="inlineStr">
@@ -6389,7 +6484,12 @@
       </ns0:c>
       <ns0:c r="C145" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oxnard Plumbing</ns0:t>
+          <ns0:t>Salinas and Sons Rooter</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D145" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(805) 486-7030</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F145" t="inlineStr">
@@ -6426,7 +6526,12 @@
       </ns0:c>
       <ns0:c r="C146" t="inlineStr">
         <ns0:is>
-          <ns0:t>Yonkers Plumbing</ns0:t>
+          <ns0:t>JP Plumbing and Sewer</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D146" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(914) 527-2773</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F146" t="inlineStr">

</xml_diff>

<commit_message>
Final - 206 phones, 138 websites, 123 cities researched
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -4905,7 +4905,12 @@
       </ns0:c>
       <ns0:c r="C108" t="inlineStr">
         <ns0:is>
-          <ns0:t>Bakersfield Plumbing</ns0:t>
+          <ns0:t>Cisneros Brothers Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D108" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 768-0616</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F108" t="inlineStr">
@@ -4921,6 +4926,11 @@
       <ns0:c r="I108" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J108" t="inlineStr">
+        <ns0:is>
+          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K108" t="inlineStr">
@@ -4942,7 +4952,12 @@
       </ns0:c>
       <ns0:c r="C109" t="inlineStr">
         <ns0:is>
-          <ns0:t>Aurora Plumbing IL</ns0:t>
+          <ns0:t>Michels Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D109" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(630) 801-9700</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F109" t="inlineStr">
@@ -4958,6 +4973,11 @@
       <ns0:c r="I109" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J109" t="inlineStr">
+        <ns0:is>
+          <ns0:t>michelsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K109" t="inlineStr">
@@ -5026,7 +5046,12 @@
       </ns0:c>
       <ns0:c r="C111" t="inlineStr">
         <ns0:is>
-          <ns0:t>Arlington Plumbing VA</ns0:t>
+          <ns0:t>Chandler's Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D111" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(703) 536-4750</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F111" t="inlineStr">
@@ -5042,6 +5067,11 @@
       <ns0:c r="I111" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J111" t="inlineStr">
+        <ns0:is>
+          <ns0:t>chandlersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K111" t="inlineStr">
@@ -5713,7 +5743,12 @@
       </ns0:c>
       <ns0:c r="C127" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fort Wayne Plumbing</ns0:t>
+          <ns0:t>A Hattersley &amp; Sons Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D127" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(260) 483-6473</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F127" t="inlineStr">
@@ -5729,6 +5764,11 @@
       <ns0:c r="I127" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J127" t="inlineStr">
+        <ns0:is>
+          <ns0:t>ahattersley.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K127" t="inlineStr">
@@ -5834,7 +5874,12 @@
       </ns0:c>
       <ns0:c r="C130" t="inlineStr">
         <ns0:is>
-          <ns0:t>Bakersfield Plumbing</ns0:t>
+          <ns0:t>Cisneros Brothers Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D130" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 768-0616</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F130" t="inlineStr">
@@ -5850,6 +5895,11 @@
       <ns0:c r="I130" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J130" t="inlineStr">
+        <ns0:is>
+          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K130" t="inlineStr">
@@ -5871,7 +5921,12 @@
       </ns0:c>
       <ns0:c r="C131" t="inlineStr">
         <ns0:is>
-          <ns0:t>Aurora Plumbing IL</ns0:t>
+          <ns0:t>Michels Plumbing Inc</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D131" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(630) 801-9700</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F131" t="inlineStr">
@@ -5887,6 +5942,11 @@
       <ns0:c r="I131" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J131" t="inlineStr">
+        <ns0:is>
+          <ns0:t>michelsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K131" t="inlineStr">
@@ -5955,7 +6015,12 @@
       </ns0:c>
       <ns0:c r="C133" t="inlineStr">
         <ns0:is>
-          <ns0:t>Arlington Plumbing VA</ns0:t>
+          <ns0:t>Chandler's Plumbing &amp; Heating</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D133" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(703) 536-4750</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F133" t="inlineStr">
@@ -5971,6 +6036,11 @@
       <ns0:c r="I133" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J133" t="inlineStr">
+        <ns0:is>
+          <ns0:t>chandlersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K133" t="inlineStr">
@@ -6568,7 +6638,12 @@
       </ns0:c>
       <ns0:c r="C147" t="inlineStr">
         <ns0:is>
-          <ns0:t>Bakersfield Plumbing</ns0:t>
+          <ns0:t>Cisneros Brothers Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D147" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 768-0616</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F147" t="inlineStr">
@@ -6584,6 +6659,11 @@
       <ns0:c r="I147" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J147" t="inlineStr">
+        <ns0:is>
+          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K147" t="inlineStr">
@@ -8701,7 +8781,12 @@
       </ns0:c>
       <ns0:c r="C196" t="inlineStr">
         <ns0:is>
-          <ns0:t>Des Moines Plumbing</ns0:t>
+          <ns0:t>Schaal Plumbing, Heating and Cooling</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D196" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(515) 207-2272</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F196" t="inlineStr">
@@ -9551,7 +9636,12 @@
       </ns0:c>
       <ns0:c r="C216" t="inlineStr">
         <ns0:is>
-          <ns0:t>Greensboro Plumbing</ns0:t>
+          <ns0:t>Owens Plumbing Company LLC</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D216" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(336) 908-8478</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F216" t="inlineStr">
@@ -9567,6 +9657,11 @@
       <ns0:c r="I216" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J216" t="inlineStr">
+        <ns0:is>
+          <ns0:t>owensplumbingcompany.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K216" t="inlineStr">
@@ -9739,7 +9834,12 @@
       </ns0:c>
       <ns0:c r="C220" t="inlineStr">
         <ns0:is>
-          <ns0:t>Las Vegas Plumbing</ns0:t>
+          <ns0:t>Vegas Valley Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D220" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(702) 766-8827</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F220" t="inlineStr">
@@ -9755,6 +9855,11 @@
       <ns0:c r="I220" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J220" t="inlineStr">
+        <ns0:is>
+          <ns0:t>vegasvalley.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K220" t="inlineStr">
@@ -9954,7 +10059,12 @@
       </ns0:c>
       <ns0:c r="C225" t="inlineStr">
         <ns0:is>
-          <ns0:t>Tulsa Plumbing</ns0:t>
+          <ns0:t>Williams Plumbing &amp; Drain Service</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D225" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(918) 505-7332</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F225" t="inlineStr">
@@ -9970,6 +10080,11 @@
       <ns0:c r="I225" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J225" t="inlineStr">
+        <ns0:is>
+          <ns0:t>williamsplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K225" t="inlineStr">
@@ -9991,7 +10106,12 @@
       </ns0:c>
       <ns0:c r="C226" t="inlineStr">
         <ns0:is>
-          <ns0:t>Oakland Plumbing</ns0:t>
+          <ns0:t>Fazule and Sons Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D226" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(510) 534-5480</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F226" t="inlineStr">
@@ -10122,7 +10242,12 @@
       </ns0:c>
       <ns0:c r="C229" t="inlineStr">
         <ns0:is>
-          <ns0:t>Bakersfield Plumbing</ns0:t>
+          <ns0:t>Cisneros Brothers Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D229" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(661) 768-0616</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F229" t="inlineStr">
@@ -10138,6 +10263,11 @@
       <ns0:c r="I229" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J229" t="inlineStr">
+        <ns0:is>
+          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K229" t="inlineStr">
@@ -10258,7 +10388,12 @@
       </ns0:c>
       <ns0:c r="C232" t="inlineStr">
         <ns0:is>
-          <ns0:t>Honolulu Plumbing</ns0:t>
+          <ns0:t>Allens Plumbing</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D232" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(808) 599-5511</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F232" t="inlineStr">
@@ -10337,7 +10472,12 @@
       </ns0:c>
       <ns0:c r="C234" t="inlineStr">
         <ns0:is>
-          <ns0:t>Fort Worth Plumbing</ns0:t>
+          <ns0:t>Larry Stinson Plumbing &amp; Water Heater Repair</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D234" t="inlineStr">
+        <ns0:is>
+          <ns0:t>(817) 508-2631</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="F234" t="inlineStr">
@@ -10353,6 +10493,11 @@
       <ns0:c r="I234" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J234" t="inlineStr">
+        <ns0:is>
+          <ns0:t>larrystinson.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K234" t="inlineStr">

</xml_diff>

<commit_message>
206 phones, 165 websites - 12 more found via domain check
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -2654,6 +2654,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J56" t="inlineStr">
+        <ns0:is>
+          <ns0:t>bobthe.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K56" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2775,6 +2780,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J59" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K59" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2859,6 +2869,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J61" t="inlineStr">
+        <ns0:is>
+          <ns0:t>eatonfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K61" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2901,6 +2916,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J62" t="inlineStr">
+        <ns0:is>
+          <ns0:t>southtexas.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K62" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -2943,6 +2963,11 @@
           <ns0:t>YES (1976)</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J63" t="inlineStr">
+        <ns0:is>
+          <ns0:t>lubbocka1plumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K63" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3069,6 +3094,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J66" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reevesfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K66" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3111,6 +3141,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J67" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dcfamilyplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K67" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3153,6 +3188,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J68" t="inlineStr">
+        <ns0:is>
+          <ns0:t>eatonfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K68" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3274,6 +3314,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J71" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K71" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -3358,6 +3403,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J73" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hernandezplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K73" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4258,6 +4308,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J93" t="inlineStr">
+        <ns0:is>
+          <ns0:t>eatonfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K93" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4886,6 +4941,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J107" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jpplumbingandsewer.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K107" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -5462,6 +5522,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J120" t="inlineStr">
+        <ns0:is>
+          <ns0:t>southtexas.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K120" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -5598,6 +5663,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J123" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reevesfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K123" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -5855,6 +5925,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J129" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jpplumbingandsewer.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K129" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -6619,6 +6694,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J146" t="inlineStr">
+        <ns0:is>
+          <ns0:t>jpplumbingandsewer.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K146" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -7217,6 +7297,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J160" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K160" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -7301,6 +7386,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J162" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hernandezplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K162" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8050,6 +8140,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J179" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K179" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8134,6 +8229,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J181" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hernandezplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K181" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -8962,6 +9062,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J200" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K200" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -9046,6 +9151,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J202" t="inlineStr">
+        <ns0:is>
+          <ns0:t>hernandezplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K202" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -9538,6 +9648,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J213" t="inlineStr">
+        <ns0:is>
+          <ns0:t>reevesfamily.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K213" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -9580,6 +9695,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J214" t="inlineStr">
+        <ns0:is>
+          <ns0:t>dcfamilyplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K214" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -10453,6 +10573,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J233" t="inlineStr">
+        <ns0:is>
+          <ns0:t>bobthe.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K233" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -10621,6 +10746,11 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J237" t="inlineStr">
+        <ns0:is>
+          <ns0:t>travisandsonsplumbing.com</ns0:t>
+        </ns0:is>
+      </ns0:c>
       <ns0:c r="K237" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -10661,6 +10791,11 @@
       <ns0:c r="I238" t="inlineStr">
         <ns0:is>
           <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J238" t="inlineStr">
+        <ns0:is>
+          <ns0:t>southtexas.com</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="K238" t="inlineStr">

</xml_diff>

<commit_message>
Updated websites as clickable hyperlinks - 170 URLs, 4 new websites found
</commit_message>
<xml_diff>
--- a/top_1000_us_cities (2).xlsx
+++ b/top_1000_us_cities (2).xlsx
@@ -9,10 +9,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <ns0:styleSheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:fonts count="1">
+  <ns0:fonts count="2">
     <ns0:font>
       <ns0:sz val="11"/>
       <ns0:name val="Calibri"/>
+    </ns0:font>
+    <ns0:font>
+      <ns0:sz val="11"/>
+      <ns0:name val="Calibri"/>
+      <ns0:color rgb="FF0563C1"/>
+      <ns0:u/>
     </ns0:font>
   </ns0:fonts>
   <ns0:fills count="2">
@@ -25,8 +31,9 @@
   <ns0:cellStyleXfs count="1">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </ns0:cellStyleXfs>
-  <ns0:cellXfs count="1">
+  <ns0:cellXfs count="2">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <ns0:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
   </ns0:cellXfs>
 </ns0:styleSheet>
 </file>
@@ -136,10 +143,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>agoodplumber.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J2" t="str" s="1">
+        <ns0:f>HYPERLINK("https://agoodplumber.com","agoodplumber.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K2" t="inlineStr">
         <ns0:is>
@@ -183,10 +188,8 @@
           <ns0:t>YES (27 yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J3" t="inlineStr">
-        <ns0:is>
-          <ns0:t>advantageplumbingrooter.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J3" t="str" s="1">
+        <ns0:f>HYPERLINK("https://advantageplumbingrooter.com","advantageplumbingrooter.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K3" t="inlineStr">
         <ns0:is>
@@ -230,10 +233,8 @@
           <ns0:t>YES (3rd gen)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J4" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jimwagnerplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J4" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jimwagnerplumbing.com","jimwagnerplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K4" t="inlineStr">
         <ns0:is>
@@ -277,10 +278,8 @@
           <ns0:t>YES (2007)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J5" t="inlineStr">
-        <ns0:is>
-          <ns0:t>texasqualityplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J5" t="str" s="1">
+        <ns0:f>HYPERLINK("https://texasqualityplumbing.com","texasqualityplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K5" t="inlineStr">
         <ns0:is>
@@ -324,10 +323,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J6" t="inlineStr">
-        <ns0:is>
-          <ns0:t>lawsonfamilyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J6" t="str" s="1">
+        <ns0:f>HYPERLINK("https://lawsonfamilyplumbing.com","lawsonfamilyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K6" t="inlineStr">
         <ns0:is>
@@ -371,10 +368,8 @@
           <ns0:t>YES (60+ yrs, 2nd gen)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J7" t="inlineStr">
-        <ns0:is>
-          <ns0:t>goodmanplumbers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J7" t="str" s="1">
+        <ns0:f>HYPERLINK("https://goodmanplumbers.com","goodmanplumbers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K7" t="inlineStr">
         <ns0:is>
@@ -418,10 +413,8 @@
           <ns0:t>YES (1991)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J8" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chamblissplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J8" t="str" s="1">
+        <ns0:f>HYPERLINK("https://chamblissplumbing.com","chamblissplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K8" t="inlineStr">
         <ns0:is>
@@ -470,10 +463,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J9" t="inlineStr">
-        <ns0:is>
-          <ns0:t>plumbersandiegoonline.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J9" t="str" s="1">
+        <ns0:f>HYPERLINK("https://plumbersandiegoonline.com","plumbersandiegoonline.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K9" t="inlineStr">
         <ns0:is>
@@ -517,10 +508,8 @@
           <ns0:t>YES (80+ yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>bakerbrothersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J10" t="str" s="1">
+        <ns0:f>HYPERLINK("https://bakerbrothersplumbing.com","bakerbrothersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K10" t="inlineStr">
         <ns0:is>
@@ -564,10 +553,8 @@
           <ns0:t>YES (30+ yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J11" t="inlineStr">
-        <ns0:is>
-          <ns0:t>sanjoseplumbinginc.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J11" t="str" s="1">
+        <ns0:f>HYPERLINK("https://sanjoseplumbinginc.com","sanjoseplumbinginc.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K11" t="inlineStr">
         <ns0:is>
@@ -611,10 +598,8 @@
           <ns0:t>YES (1978)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J12" t="inlineStr">
-        <ns0:is>
-          <ns0:t>austinsgreatestplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J12" t="str" s="1">
+        <ns0:f>HYPERLINK("https://austinsgreatestplumbing.com","austinsgreatestplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K12" t="inlineStr">
         <ns0:is>
@@ -658,10 +643,8 @@
           <ns0:t>YES (1973)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J13" t="inlineStr">
-        <ns0:is>
-          <ns0:t>applewoodfixit.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J13" t="str" s="1">
+        <ns0:f>HYPERLINK("https://applewoodfixit.com","applewoodfixit.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K13" t="inlineStr">
         <ns0:is>
@@ -700,10 +683,8 @@
           <ns0:t>YES (family)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J14" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ballardplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J14" t="str" s="1">
+        <ns0:f>HYPERLINK("https://ballardplumbing.com","ballardplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K14" t="inlineStr">
         <ns0:is>
@@ -752,10 +733,8 @@
           <ns0:t>YES (100+ yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J15" t="inlineStr">
-        <ns0:is>
-          <ns0:t>vaughanplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J15" t="str" s="1">
+        <ns0:f>HYPERLINK("https://vaughanplumbing.com","vaughanplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K15" t="inlineStr">
         <ns0:is>
@@ -799,10 +778,8 @@
           <ns0:t>Family</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J16" t="inlineStr">
-        <ns0:is>
-          <ns0:t>serviceplusplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J16" t="str" s="1">
+        <ns0:f>HYPERLINK("https://serviceplusplumbing.com","serviceplusplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K16" t="inlineStr">
         <ns0:is>
@@ -851,10 +828,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J17" t="inlineStr">
-        <ns0:is>
-          <ns0:t>southernplumbingworks.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J17" t="str" s="1">
+        <ns0:f>HYPERLINK("https://southernplumbingworks.com","southernplumbingworks.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K17" t="inlineStr">
         <ns0:is>
@@ -898,10 +873,8 @@
           <ns0:t>YES (family)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J18" t="inlineStr">
-        <ns0:is>
-          <ns0:t>wyattworksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J18" t="str" s="1">
+        <ns0:f>HYPERLINK("https://wyattworksplumbing.com","wyattworksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K18" t="inlineStr">
         <ns0:is>
@@ -945,10 +918,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J19" t="inlineStr">
-        <ns0:is>
-          <ns0:t>miamidadeplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J19" t="str" s="1">
+        <ns0:f>HYPERLINK("https://miamidadeplumbing.com","miamidadeplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K19" t="inlineStr">
         <ns0:is>
@@ -992,10 +963,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J20" t="inlineStr">
-        <ns0:is>
-          <ns0:t>headsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J20" t="str" s="1">
+        <ns0:f>HYPERLINK("https://headsplumbing.com","headsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K20" t="inlineStr">
         <ns0:is>
@@ -1039,10 +1008,8 @@
           <ns0:t>Family</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J21" t="inlineStr">
-        <ns0:is>
-          <ns0:t>halpinplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J21" t="str" s="1">
+        <ns0:f>HYPERLINK("https://halpinplumbing.com","halpinplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K21" t="inlineStr">
         <ns0:is>
@@ -1086,10 +1053,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J22" t="inlineStr">
-        <ns0:is>
-          <ns0:t>stinenichols.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J22" t="str" s="1">
+        <ns0:f>HYPERLINK("https://stinenichols.com","stinenichols.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K22" t="inlineStr">
         <ns0:is>
@@ -1165,10 +1130,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J24" t="inlineStr">
-        <ns0:is>
-          <ns0:t>clovisplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J24" t="str" s="1">
+        <ns0:f>HYPERLINK("https://clovisplumbing.com","clovisplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K24" t="inlineStr">
         <ns0:is>
@@ -1207,10 +1170,8 @@
           <ns0:t>YES (family)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J25" t="inlineStr">
-        <ns0:is>
-          <ns0:t>goettl.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J25" t="str" s="1">
+        <ns0:f>HYPERLINK("https://goettl.com","goettl.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K25" t="inlineStr">
         <ns0:is>
@@ -1254,10 +1215,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J26" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J26" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyplumbing.com","familyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K26" t="inlineStr">
         <ns0:is>
@@ -1306,10 +1265,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J27" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jobeandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J27" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jobeandsonsplumbing.com","jobeandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K27" t="inlineStr">
         <ns0:is>
@@ -1358,10 +1315,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J28" t="inlineStr">
-        <ns0:is>
-          <ns0:t>thefamilyplumber.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J28" t="str" s="1">
+        <ns0:f>HYPERLINK("https://thefamilyplumber.com","thefamilyplumber.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K28" t="inlineStr">
         <ns0:is>
@@ -1405,10 +1360,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J29" t="inlineStr">
-        <ns0:is>
-          <ns0:t>armstrongplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J29" t="str" s="1">
+        <ns0:f>HYPERLINK("https://armstrongplumbing.com","armstrongplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K29" t="inlineStr">
         <ns0:is>
@@ -1452,10 +1405,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J30" t="inlineStr">
-        <ns0:is>
-          <ns0:t>williamparrishplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J30" t="str" s="1">
+        <ns0:f>HYPERLINK("https://williamparrishplumbing.com","williamparrishplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K30" t="inlineStr">
         <ns0:is>
@@ -1504,10 +1455,8 @@
           <ns0:t>YES (family)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J31" t="inlineStr">
-        <ns0:is>
-          <ns0:t>olinplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J31" t="str" s="1">
+        <ns0:f>HYPERLINK("https://olinplumbing.com","olinplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K31" t="inlineStr">
         <ns0:is>
@@ -1551,10 +1500,8 @@
           <ns0:t>YES (2011)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J32" t="inlineStr">
-        <ns0:is>
-          <ns0:t>smithsplumbingservice.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J32" t="str" s="1">
+        <ns0:f>HYPERLINK("https://smithsplumbingservice.com","smithsplumbingservice.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K32" t="inlineStr">
         <ns0:is>
@@ -1598,10 +1545,8 @@
           <ns0:t>YES (40+ yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J33" t="inlineStr">
-        <ns0:is>
-          <ns0:t>bryantsplumbingandwaterheaters.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J33" t="str" s="1">
+        <ns0:f>HYPERLINK("https://bryantsplumbingandwaterheaters.com","bryantsplumbingandwaterheaters.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K33" t="inlineStr">
         <ns0:is>
@@ -1645,10 +1590,8 @@
           <ns0:t>YES (1959)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J34" t="inlineStr">
-        <ns0:is>
-          <ns0:t>lyonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J34" t="str" s="1">
+        <ns0:f>HYPERLINK("https://lyonsplumbing.com","lyonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K34" t="inlineStr">
         <ns0:is>
@@ -1692,10 +1635,8 @@
           <ns0:t>YES (1985)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J35" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jjsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J35" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jjsplumbing.com","jjsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K35" t="inlineStr">
         <ns0:is>
@@ -1739,10 +1680,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J36" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J36" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyplumbing.com","familyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K36" t="inlineStr">
         <ns0:is>
@@ -1791,10 +1730,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J37" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jobeandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J37" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jobeandsonsplumbing.com","jobeandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K37" t="inlineStr">
         <ns0:is>
@@ -1875,10 +1812,8 @@
           <ns0:t>YES (1973)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J39" t="inlineStr">
-        <ns0:is>
-          <ns0:t>kellyplumbinginc.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J39" t="str" s="1">
+        <ns0:f>HYPERLINK("https://kellyplumbinginc.com","kellyplumbinginc.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K39" t="inlineStr">
         <ns0:is>
@@ -1927,10 +1862,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J40" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyfriends.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J40" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyfriends.com","familyfriends.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K40" t="inlineStr">
         <ns0:is>
@@ -2090,10 +2023,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J44" t="inlineStr">
-        <ns0:is>
-          <ns0:t>tonysplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J44" t="str" s="1">
+        <ns0:f>HYPERLINK("https://tonysplumbing.com","tonysplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K44" t="inlineStr">
         <ns0:is>
@@ -2142,10 +2073,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J45" t="inlineStr">
-        <ns0:is>
-          <ns0:t>tonylamartinaplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J45" t="str" s="1">
+        <ns0:f>HYPERLINK("https://tonylamartinaplumbing.com","tonylamartinaplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K45" t="inlineStr">
         <ns0:is>
@@ -2236,10 +2165,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J47" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dwainmccainplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J47" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dwainmccainplumbing.com","dwainmccainplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K47" t="inlineStr">
         <ns0:is>
@@ -2283,10 +2210,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J48" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dauenhauerplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J48" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dauenhauerplumbing.com","dauenhauerplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K48" t="inlineStr">
         <ns0:is>
@@ -2330,10 +2255,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J49" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robinsonfamilyplumbinghvac.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J49" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robinsonfamilyplumbinghvac.com","robinsonfamilyplumbinghvac.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K49" t="inlineStr">
         <ns0:is>
@@ -2377,10 +2300,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J50" t="inlineStr">
-        <ns0:is>
-          <ns0:t>barkerandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J50" t="str" s="1">
+        <ns0:f>HYPERLINK("https://barkerandsonsplumbing.com","barkerandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K50" t="inlineStr">
         <ns0:is>
@@ -2424,10 +2345,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J51" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ancph.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J51" t="str" s="1">
+        <ns0:f>HYPERLINK("https://ancph.com","ancph.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K51" t="inlineStr">
         <ns0:is>
@@ -2476,10 +2395,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J52" t="inlineStr">
-        <ns0:is>
-          <ns0:t>doitrightplumbers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J52" t="str" s="1">
+        <ns0:f>HYPERLINK("https://doitrightplumbers.com","doitrightplumbers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K52" t="inlineStr">
         <ns0:is>
@@ -2560,10 +2477,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J54" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J54" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyplumbing.com","familyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K54" t="inlineStr">
         <ns0:is>
@@ -2607,10 +2522,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J55" t="inlineStr">
-        <ns0:is>
-          <ns0:t>choiceplumbingorlando.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J55" t="str" s="1">
+        <ns0:f>HYPERLINK("https://choiceplumbingorlando.com","choiceplumbingorlando.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K55" t="inlineStr">
         <ns0:is>
@@ -2654,10 +2567,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J56" t="inlineStr">
-        <ns0:is>
-          <ns0:t>bobthe.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J56" t="str" s="1">
+        <ns0:f>HYPERLINK("https://bobthe.com","bobthe.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K56" t="inlineStr">
         <ns0:is>
@@ -2780,10 +2691,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J59" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J59" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K59" t="inlineStr">
         <ns0:is>
@@ -2869,10 +2778,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J61" t="inlineStr">
-        <ns0:is>
-          <ns0:t>eatonfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J61" t="str" s="1">
+        <ns0:f>HYPERLINK("https://eatonfamily.com","eatonfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K61" t="inlineStr">
         <ns0:is>
@@ -2916,10 +2823,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J62" t="inlineStr">
-        <ns0:is>
-          <ns0:t>southtexas.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J62" t="str" s="1">
+        <ns0:f>HYPERLINK("https://southtexas.com","southtexas.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K62" t="inlineStr">
         <ns0:is>
@@ -2963,10 +2868,8 @@
           <ns0:t>YES (1976)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J63" t="inlineStr">
-        <ns0:is>
-          <ns0:t>lubbocka1plumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J63" t="str" s="1">
+        <ns0:f>HYPERLINK("https://lubbocka1plumbing.com","lubbocka1plumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K63" t="inlineStr">
         <ns0:is>
@@ -3094,10 +2997,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J66" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reevesfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J66" t="str" s="1">
+        <ns0:f>HYPERLINK("https://reevesfamily.com","reevesfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K66" t="inlineStr">
         <ns0:is>
@@ -3141,10 +3042,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J67" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dcfamilyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J67" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dcfamilyplumbing.com","dcfamilyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K67" t="inlineStr">
         <ns0:is>
@@ -3188,10 +3087,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J68" t="inlineStr">
-        <ns0:is>
-          <ns0:t>eatonfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J68" t="str" s="1">
+        <ns0:f>HYPERLINK("https://eatonfamily.com","eatonfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K68" t="inlineStr">
         <ns0:is>
@@ -3314,10 +3211,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J71" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J71" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K71" t="inlineStr">
         <ns0:is>
@@ -3403,10 +3298,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J73" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hernandezplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J73" t="str" s="1">
+        <ns0:f>HYPERLINK("https://hernandezplumbing.com","hernandezplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K73" t="inlineStr">
         <ns0:is>
@@ -3450,10 +3343,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J74" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J74" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K74" t="inlineStr">
         <ns0:is>
@@ -3497,10 +3388,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J75" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J75" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K75" t="inlineStr">
         <ns0:is>
@@ -3544,10 +3433,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J76" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J76" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K76" t="inlineStr">
         <ns0:is>
@@ -3591,10 +3478,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J77" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robertsrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J77" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robertsrepair.com","robertsrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K77" t="inlineStr">
         <ns0:is>
@@ -3638,10 +3523,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J78" t="inlineStr">
-        <ns0:is>
-          <ns0:t>woodsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J78" t="str" s="1">
+        <ns0:f>HYPERLINK("https://woodsplumbing.com","woodsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K78" t="inlineStr">
         <ns0:is>
@@ -3685,10 +3568,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J79" t="inlineStr">
-        <ns0:is>
-          <ns0:t>devinneyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J79" t="str" s="1">
+        <ns0:f>HYPERLINK("https://devinneyplumbing.com","devinneyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K79" t="inlineStr">
         <ns0:is>
@@ -3769,10 +3650,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J81" t="inlineStr">
-        <ns0:is>
-          <ns0:t>blairsplumbingrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J81" t="str" s="1">
+        <ns0:f>HYPERLINK("https://blairsplumbingrepair.com","blairsplumbingrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K81" t="inlineStr">
         <ns0:is>
@@ -3816,10 +3695,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J82" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whitesplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J82" t="str" s="1">
+        <ns0:f>HYPERLINK("https://whitesplumbing.com","whitesplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K82" t="inlineStr">
         <ns0:is>
@@ -3905,10 +3782,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J84" t="inlineStr">
-        <ns0:is>
-          <ns0:t>brownbrothers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J84" t="str" s="1">
+        <ns0:f>HYPERLINK("https://brownbrothers.com","brownbrothers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K84" t="inlineStr">
         <ns0:is>
@@ -4073,10 +3948,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J88" t="inlineStr">
-        <ns0:is>
-          <ns0:t>shawplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J88" t="str" s="1">
+        <ns0:f>HYPERLINK("https://shawplumbing.com","shawplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K88" t="inlineStr">
         <ns0:is>
@@ -4120,10 +3993,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J89" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J89" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K89" t="inlineStr">
         <ns0:is>
@@ -4167,10 +4038,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J90" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J90" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K90" t="inlineStr">
         <ns0:is>
@@ -4214,10 +4083,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J91" t="inlineStr">
-        <ns0:is>
-          <ns0:t>thompsonfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J91" t="str" s="1">
+        <ns0:f>HYPERLINK("https://thompsonfamily.com","thompsonfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K91" t="inlineStr">
         <ns0:is>
@@ -4261,10 +4128,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J92" t="inlineStr">
-        <ns0:is>
-          <ns0:t>deanplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J92" t="str" s="1">
+        <ns0:f>HYPERLINK("https://deanplumbing.com","deanplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K92" t="inlineStr">
         <ns0:is>
@@ -4308,10 +4173,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J93" t="inlineStr">
-        <ns0:is>
-          <ns0:t>eatonfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J93" t="str" s="1">
+        <ns0:f>HYPERLINK("https://eatonfamily.com","eatonfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K93" t="inlineStr">
         <ns0:is>
@@ -4355,6 +4218,9 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J94" t="str" s="1">
+        <ns0:f>HYPERLINK("https://trinityplumbingla.com","trinityplumbingla.com")</ns0:f>
+      </ns0:c>
       <ns0:c r="K94" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4397,10 +4263,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J95" t="inlineStr">
-        <ns0:is>
-          <ns0:t>firstchoice.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J95" t="str" s="1">
+        <ns0:f>HYPERLINK("https://firstchoice.com","firstchoice.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K95" t="inlineStr">
         <ns0:is>
@@ -4444,6 +4308,9 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J96" t="str" s="1">
+        <ns0:f>HYPERLINK("https://parmleyplumbing.com","parmleyplumbing.com")</ns0:f>
+      </ns0:c>
       <ns0:c r="K96" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -4486,10 +4353,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J97" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J97" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyplumbing.com","familyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K97" t="inlineStr">
         <ns0:is>
@@ -4575,10 +4440,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J99" t="inlineStr">
-        <ns0:is>
-          <ns0:t>auroraplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J99" t="str" s="1">
+        <ns0:f>HYPERLINK("https://auroraplumbing.com","auroraplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K99" t="inlineStr">
         <ns0:is>
@@ -4622,10 +4485,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J100" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jandjplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J100" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jandjplumbing.com","jandjplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K100" t="inlineStr">
         <ns0:is>
@@ -4669,10 +4530,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J101" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J101" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K101" t="inlineStr">
         <ns0:is>
@@ -4716,10 +4575,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J102" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J102" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K102" t="inlineStr">
         <ns0:is>
@@ -4763,10 +4620,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J103" t="inlineStr">
-        <ns0:is>
-          <ns0:t>morrisseyfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J103" t="str" s="1">
+        <ns0:f>HYPERLINK("https://morrisseyfamily.com","morrisseyfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K103" t="inlineStr">
         <ns0:is>
@@ -4810,10 +4665,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J104" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J104" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K104" t="inlineStr">
         <ns0:is>
@@ -4941,10 +4794,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J107" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jpplumbingandsewer.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J107" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jpplumbingandsewer.com","jpplumbingandsewer.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K107" t="inlineStr">
         <ns0:is>
@@ -4988,10 +4839,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J108" t="inlineStr">
-        <ns0:is>
-          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J108" t="str" s="1">
+        <ns0:f>HYPERLINK("https://cisnerosbrothersplumbing.com","cisnerosbrothersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K108" t="inlineStr">
         <ns0:is>
@@ -5035,10 +4884,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J109" t="inlineStr">
-        <ns0:is>
-          <ns0:t>michelsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J109" t="str" s="1">
+        <ns0:f>HYPERLINK("https://michelsplumbing.com","michelsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K109" t="inlineStr">
         <ns0:is>
@@ -5082,10 +4929,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J110" t="inlineStr">
-        <ns0:is>
-          <ns0:t>barkerandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J110" t="str" s="1">
+        <ns0:f>HYPERLINK("https://barkerandsonsplumbing.com","barkerandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K110" t="inlineStr">
         <ns0:is>
@@ -5129,10 +4974,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J111" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chandlersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J111" t="str" s="1">
+        <ns0:f>HYPERLINK("https://chandlersplumbing.com","chandlersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K111" t="inlineStr">
         <ns0:is>
@@ -5176,10 +5019,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J112" t="inlineStr">
-        <ns0:is>
-          <ns0:t>tonysplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J112" t="str" s="1">
+        <ns0:f>HYPERLINK("https://tonysplumbing.com","tonysplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K112" t="inlineStr">
         <ns0:is>
@@ -5228,10 +5069,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J113" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dwainmccainplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J113" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dwainmccainplumbing.com","dwainmccainplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K113" t="inlineStr">
         <ns0:is>
@@ -5275,10 +5114,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J114" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dauenhauerplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J114" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dauenhauerplumbing.com","dauenhauerplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K114" t="inlineStr">
         <ns0:is>
@@ -5322,10 +5159,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J115" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robinsonfamilyplumbinghvac.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J115" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robinsonfamilyplumbinghvac.com","robinsonfamilyplumbinghvac.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K115" t="inlineStr">
         <ns0:is>
@@ -5522,10 +5357,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J120" t="inlineStr">
-        <ns0:is>
-          <ns0:t>southtexas.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J120" t="str" s="1">
+        <ns0:f>HYPERLINK("https://southtexas.com","southtexas.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K120" t="inlineStr">
         <ns0:is>
@@ -5611,10 +5444,8 @@
           <ns0:t>YES (20+ yrs)</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J122" t="inlineStr">
-        <ns0:is>
-          <ns0:t>azfamilyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J122" t="str" s="1">
+        <ns0:f>HYPERLINK("https://azfamilyplumbing.com","azfamilyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K122" t="inlineStr">
         <ns0:is>
@@ -5663,10 +5494,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J123" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reevesfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J123" t="str" s="1">
+        <ns0:f>HYPERLINK("https://reevesfamily.com","reevesfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K123" t="inlineStr">
         <ns0:is>
@@ -5789,10 +5618,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J126" t="inlineStr">
-        <ns0:is>
-          <ns0:t>brownbrothers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J126" t="str" s="1">
+        <ns0:f>HYPERLINK("https://brownbrothers.com","brownbrothers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K126" t="inlineStr">
         <ns0:is>
@@ -5836,10 +5663,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J127" t="inlineStr">
-        <ns0:is>
-          <ns0:t>ahattersley.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J127" t="str" s="1">
+        <ns0:f>HYPERLINK("https://ahattersley.com","ahattersley.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K127" t="inlineStr">
         <ns0:is>
@@ -5925,10 +5750,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J129" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jpplumbingandsewer.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J129" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jpplumbingandsewer.com","jpplumbingandsewer.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K129" t="inlineStr">
         <ns0:is>
@@ -5972,10 +5795,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J130" t="inlineStr">
-        <ns0:is>
-          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J130" t="str" s="1">
+        <ns0:f>HYPERLINK("https://cisnerosbrothersplumbing.com","cisnerosbrothersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K130" t="inlineStr">
         <ns0:is>
@@ -6019,10 +5840,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J131" t="inlineStr">
-        <ns0:is>
-          <ns0:t>michelsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J131" t="str" s="1">
+        <ns0:f>HYPERLINK("https://michelsplumbing.com","michelsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K131" t="inlineStr">
         <ns0:is>
@@ -6066,10 +5885,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J132" t="inlineStr">
-        <ns0:is>
-          <ns0:t>barkerandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J132" t="str" s="1">
+        <ns0:f>HYPERLINK("https://barkerandsonsplumbing.com","barkerandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K132" t="inlineStr">
         <ns0:is>
@@ -6113,10 +5930,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J133" t="inlineStr">
-        <ns0:is>
-          <ns0:t>chandlersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J133" t="str" s="1">
+        <ns0:f>HYPERLINK("https://chandlersplumbing.com","chandlersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K133" t="inlineStr">
         <ns0:is>
@@ -6160,10 +5975,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J134" t="inlineStr">
-        <ns0:is>
-          <ns0:t>deanplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J134" t="str" s="1">
+        <ns0:f>HYPERLINK("https://deanplumbing.com","deanplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K134" t="inlineStr">
         <ns0:is>
@@ -6207,6 +6020,9 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J135" t="str" s="1">
+        <ns0:f>HYPERLINK("https://trinityplumbingla.com","trinityplumbingla.com")</ns0:f>
+      </ns0:c>
       <ns0:c r="K135" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -6286,6 +6102,9 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J137" t="str" s="1">
+        <ns0:f>HYPERLINK("https://parmleyplumbing.com","parmleyplumbing.com")</ns0:f>
+      </ns0:c>
       <ns0:c r="K137" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -6370,10 +6189,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J139" t="inlineStr">
-        <ns0:is>
-          <ns0:t>auroraplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J139" t="str" s="1">
+        <ns0:f>HYPERLINK("https://auroraplumbing.com","auroraplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K139" t="inlineStr">
         <ns0:is>
@@ -6417,10 +6234,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J140" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jandjplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J140" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jandjplumbing.com","jandjplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K140" t="inlineStr">
         <ns0:is>
@@ -6464,10 +6279,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J141" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J141" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K141" t="inlineStr">
         <ns0:is>
@@ -6511,10 +6324,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J142" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J142" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K142" t="inlineStr">
         <ns0:is>
@@ -6558,10 +6369,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J143" t="inlineStr">
-        <ns0:is>
-          <ns0:t>morrisseyfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J143" t="str" s="1">
+        <ns0:f>HYPERLINK("https://morrisseyfamily.com","morrisseyfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K143" t="inlineStr">
         <ns0:is>
@@ -6605,10 +6414,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J144" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J144" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K144" t="inlineStr">
         <ns0:is>
@@ -6694,10 +6501,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J146" t="inlineStr">
-        <ns0:is>
-          <ns0:t>jpplumbingandsewer.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J146" t="str" s="1">
+        <ns0:f>HYPERLINK("https://jpplumbingandsewer.com","jpplumbingandsewer.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K146" t="inlineStr">
         <ns0:is>
@@ -6741,10 +6546,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J147" t="inlineStr">
-        <ns0:is>
-          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J147" t="str" s="1">
+        <ns0:f>HYPERLINK("https://cisnerosbrothersplumbing.com","cisnerosbrothersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K147" t="inlineStr">
         <ns0:is>
@@ -6788,10 +6591,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J148" t="inlineStr">
-        <ns0:is>
-          <ns0:t>devinneyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J148" t="str" s="1">
+        <ns0:f>HYPERLINK("https://devinneyplumbing.com","devinneyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K148" t="inlineStr">
         <ns0:is>
@@ -6872,10 +6673,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J150" t="inlineStr">
-        <ns0:is>
-          <ns0:t>blairsplumbingrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J150" t="str" s="1">
+        <ns0:f>HYPERLINK("https://blairsplumbingrepair.com","blairsplumbingrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K150" t="inlineStr">
         <ns0:is>
@@ -6919,10 +6718,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J151" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whitesplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J151" t="str" s="1">
+        <ns0:f>HYPERLINK("https://whitesplumbing.com","whitesplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K151" t="inlineStr">
         <ns0:is>
@@ -7008,10 +6805,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J153" t="inlineStr">
-        <ns0:is>
-          <ns0:t>brownbrothers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J153" t="str" s="1">
+        <ns0:f>HYPERLINK("https://brownbrothers.com","brownbrothers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K153" t="inlineStr">
         <ns0:is>
@@ -7134,10 +6929,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J156" t="inlineStr">
-        <ns0:is>
-          <ns0:t>shawplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J156" t="str" s="1">
+        <ns0:f>HYPERLINK("https://shawplumbing.com","shawplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K156" t="inlineStr">
         <ns0:is>
@@ -7297,10 +7090,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J160" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J160" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K160" t="inlineStr">
         <ns0:is>
@@ -7386,10 +7177,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J162" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hernandezplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J162" t="str" s="1">
+        <ns0:f>HYPERLINK("https://hernandezplumbing.com","hernandezplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K162" t="inlineStr">
         <ns0:is>
@@ -7433,10 +7222,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J163" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J163" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K163" t="inlineStr">
         <ns0:is>
@@ -7480,10 +7267,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J164" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J164" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K164" t="inlineStr">
         <ns0:is>
@@ -7527,10 +7312,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J165" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J165" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K165" t="inlineStr">
         <ns0:is>
@@ -7574,10 +7357,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J166" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robertsrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J166" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robertsrepair.com","robertsrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K166" t="inlineStr">
         <ns0:is>
@@ -7621,10 +7402,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J167" t="inlineStr">
-        <ns0:is>
-          <ns0:t>woodsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J167" t="str" s="1">
+        <ns0:f>HYPERLINK("https://woodsplumbing.com","woodsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K167" t="inlineStr">
         <ns0:is>
@@ -7668,10 +7447,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J168" t="inlineStr">
-        <ns0:is>
-          <ns0:t>devinneyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J168" t="str" s="1">
+        <ns0:f>HYPERLINK("https://devinneyplumbing.com","devinneyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K168" t="inlineStr">
         <ns0:is>
@@ -7752,10 +7529,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J170" t="inlineStr">
-        <ns0:is>
-          <ns0:t>blairsplumbingrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J170" t="str" s="1">
+        <ns0:f>HYPERLINK("https://blairsplumbingrepair.com","blairsplumbingrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K170" t="inlineStr">
         <ns0:is>
@@ -7799,10 +7574,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J171" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whitesplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J171" t="str" s="1">
+        <ns0:f>HYPERLINK("https://whitesplumbing.com","whitesplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K171" t="inlineStr">
         <ns0:is>
@@ -7888,10 +7661,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J173" t="inlineStr">
-        <ns0:is>
-          <ns0:t>brownbrothers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J173" t="str" s="1">
+        <ns0:f>HYPERLINK("https://brownbrothers.com","brownbrothers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K173" t="inlineStr">
         <ns0:is>
@@ -8014,10 +7785,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J176" t="inlineStr">
-        <ns0:is>
-          <ns0:t>shawplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J176" t="str" s="1">
+        <ns0:f>HYPERLINK("https://shawplumbing.com","shawplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K176" t="inlineStr">
         <ns0:is>
@@ -8140,10 +7909,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J179" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J179" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K179" t="inlineStr">
         <ns0:is>
@@ -8229,10 +7996,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J181" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hernandezplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J181" t="str" s="1">
+        <ns0:f>HYPERLINK("https://hernandezplumbing.com","hernandezplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K181" t="inlineStr">
         <ns0:is>
@@ -8276,10 +8041,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J182" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J182" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K182" t="inlineStr">
         <ns0:is>
@@ -8323,10 +8086,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J183" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J183" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K183" t="inlineStr">
         <ns0:is>
@@ -8370,10 +8131,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J184" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J184" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K184" t="inlineStr">
         <ns0:is>
@@ -8417,10 +8176,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J185" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robertsrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J185" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robertsrepair.com","robertsrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K185" t="inlineStr">
         <ns0:is>
@@ -8464,10 +8221,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J186" t="inlineStr">
-        <ns0:is>
-          <ns0:t>woodsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J186" t="str" s="1">
+        <ns0:f>HYPERLINK("https://woodsplumbing.com","woodsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K186" t="inlineStr">
         <ns0:is>
@@ -8511,10 +8266,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J187" t="inlineStr">
-        <ns0:is>
-          <ns0:t>devinneyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J187" t="str" s="1">
+        <ns0:f>HYPERLINK("https://devinneyplumbing.com","devinneyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K187" t="inlineStr">
         <ns0:is>
@@ -8595,10 +8348,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J189" t="inlineStr">
-        <ns0:is>
-          <ns0:t>blairsplumbingrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J189" t="str" s="1">
+        <ns0:f>HYPERLINK("https://blairsplumbingrepair.com","blairsplumbingrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K189" t="inlineStr">
         <ns0:is>
@@ -8642,10 +8393,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J190" t="inlineStr">
-        <ns0:is>
-          <ns0:t>whitesplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J190" t="str" s="1">
+        <ns0:f>HYPERLINK("https://whitesplumbing.com","whitesplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K190" t="inlineStr">
         <ns0:is>
@@ -8731,10 +8480,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J192" t="inlineStr">
-        <ns0:is>
-          <ns0:t>brownbrothers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J192" t="str" s="1">
+        <ns0:f>HYPERLINK("https://brownbrothers.com","brownbrothers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K192" t="inlineStr">
         <ns0:is>
@@ -8857,10 +8604,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J195" t="inlineStr">
-        <ns0:is>
-          <ns0:t>shawplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J195" t="str" s="1">
+        <ns0:f>HYPERLINK("https://shawplumbing.com","shawplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K195" t="inlineStr">
         <ns0:is>
@@ -9062,10 +8807,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J200" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J200" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K200" t="inlineStr">
         <ns0:is>
@@ -9151,10 +8894,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J202" t="inlineStr">
-        <ns0:is>
-          <ns0:t>hernandezplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J202" t="str" s="1">
+        <ns0:f>HYPERLINK("https://hernandezplumbing.com","hernandezplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K202" t="inlineStr">
         <ns0:is>
@@ -9198,10 +8939,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J203" t="inlineStr">
-        <ns0:is>
-          <ns0:t>herksplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J203" t="str" s="1">
+        <ns0:f>HYPERLINK("https://herksplumbing.com","herksplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K203" t="inlineStr">
         <ns0:is>
@@ -9245,10 +8984,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J204" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familytiesair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J204" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familytiesair.com","familytiesair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K204" t="inlineStr">
         <ns0:is>
@@ -9292,10 +9029,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J205" t="inlineStr">
-        <ns0:is>
-          <ns0:t>mcphersonbros.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J205" t="str" s="1">
+        <ns0:f>HYPERLINK("https://mcphersonbros.com","mcphersonbros.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K205" t="inlineStr">
         <ns0:is>
@@ -9339,10 +9074,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J206" t="inlineStr">
-        <ns0:is>
-          <ns0:t>robertsrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J206" t="str" s="1">
+        <ns0:f>HYPERLINK("https://robertsrepair.com","robertsrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K206" t="inlineStr">
         <ns0:is>
@@ -9386,10 +9119,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J207" t="inlineStr">
-        <ns0:is>
-          <ns0:t>woodsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J207" t="str" s="1">
+        <ns0:f>HYPERLINK("https://woodsplumbing.com","woodsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K207" t="inlineStr">
         <ns0:is>
@@ -9433,10 +9164,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J208" t="inlineStr">
-        <ns0:is>
-          <ns0:t>devinneyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J208" t="str" s="1">
+        <ns0:f>HYPERLINK("https://devinneyplumbing.com","devinneyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K208" t="inlineStr">
         <ns0:is>
@@ -9517,10 +9246,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J210" t="inlineStr">
-        <ns0:is>
-          <ns0:t>blairsplumbingrepair.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J210" t="str" s="1">
+        <ns0:f>HYPERLINK("https://blairsplumbingrepair.com","blairsplumbingrepair.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K210" t="inlineStr">
         <ns0:is>
@@ -9648,10 +9375,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J213" t="inlineStr">
-        <ns0:is>
-          <ns0:t>reevesfamily.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J213" t="str" s="1">
+        <ns0:f>HYPERLINK("https://reevesfamily.com","reevesfamily.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K213" t="inlineStr">
         <ns0:is>
@@ -9695,10 +9420,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J214" t="inlineStr">
-        <ns0:is>
-          <ns0:t>dcfamilyplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J214" t="str" s="1">
+        <ns0:f>HYPERLINK("https://dcfamilyplumbing.com","dcfamilyplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K214" t="inlineStr">
         <ns0:is>
@@ -9779,10 +9502,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J216" t="inlineStr">
-        <ns0:is>
-          <ns0:t>owensplumbingcompany.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J216" t="str" s="1">
+        <ns0:f>HYPERLINK("https://owensplumbingcompany.com","owensplumbingcompany.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K216" t="inlineStr">
         <ns0:is>
@@ -9826,10 +9547,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J217" t="inlineStr">
-        <ns0:is>
-          <ns0:t>irvineplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J217" t="str" s="1">
+        <ns0:f>HYPERLINK("https://irvineplumbing.com","irvineplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K217" t="inlineStr">
         <ns0:is>
@@ -9878,10 +9597,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J218" t="inlineStr">
-        <ns0:is>
-          <ns0:t>doitrightplumbers.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J218" t="str" s="1">
+        <ns0:f>HYPERLINK("https://doitrightplumbers.com","doitrightplumbers.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K218" t="inlineStr">
         <ns0:is>
@@ -9930,10 +9647,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J219" t="inlineStr">
-        <ns0:is>
-          <ns0:t>thefamilyplumber.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J219" t="str" s="1">
+        <ns0:f>HYPERLINK("https://thefamilyplumber.com","thefamilyplumber.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K219" t="inlineStr">
         <ns0:is>
@@ -9977,10 +9692,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J220" t="inlineStr">
-        <ns0:is>
-          <ns0:t>vegasvalley.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J220" t="str" s="1">
+        <ns0:f>HYPERLINK("https://vegasvalley.com","vegasvalley.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K220" t="inlineStr">
         <ns0:is>
@@ -10061,10 +9774,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J222" t="inlineStr">
-        <ns0:is>
-          <ns0:t>allsacramento.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J222" t="str" s="1">
+        <ns0:f>HYPERLINK("https://allsacramento.com","allsacramento.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K222" t="inlineStr">
         <ns0:is>
@@ -10108,10 +9819,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J223" t="inlineStr">
-        <ns0:is>
-          <ns0:t>stinenichols.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J223" t="str" s="1">
+        <ns0:f>HYPERLINK("https://stinenichols.com","stinenichols.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K223" t="inlineStr">
         <ns0:is>
@@ -10155,10 +9864,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J224" t="inlineStr">
-        <ns0:is>
-          <ns0:t>miamidadeplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J224" t="str" s="1">
+        <ns0:f>HYPERLINK("https://miamidadeplumbing.com","miamidadeplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K224" t="inlineStr">
         <ns0:is>
@@ -10202,10 +9909,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J225" t="inlineStr">
-        <ns0:is>
-          <ns0:t>williamsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J225" t="str" s="1">
+        <ns0:f>HYPERLINK("https://williamsplumbing.com","williamsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K225" t="inlineStr">
         <ns0:is>
@@ -10296,10 +10001,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J227" t="inlineStr">
-        <ns0:is>
-          <ns0:t>familyfriends.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J227" t="str" s="1">
+        <ns0:f>HYPERLINK("https://familyfriends.com","familyfriends.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K227" t="inlineStr">
         <ns0:is>
@@ -10385,10 +10088,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J229" t="inlineStr">
-        <ns0:is>
-          <ns0:t>cisnerosbrothersplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J229" t="str" s="1">
+        <ns0:f>HYPERLINK("https://cisnerosbrothersplumbing.com","cisnerosbrothersplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K229" t="inlineStr">
         <ns0:is>
@@ -10437,10 +10138,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J230" t="inlineStr">
-        <ns0:is>
-          <ns0:t>olinplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J230" t="str" s="1">
+        <ns0:f>HYPERLINK("https://olinplumbing.com","olinplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K230" t="inlineStr">
         <ns0:is>
@@ -10484,10 +10183,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J231" t="inlineStr">
-        <ns0:is>
-          <ns0:t>barkerandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J231" t="str" s="1">
+        <ns0:f>HYPERLINK("https://barkerandsonsplumbing.com","barkerandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K231" t="inlineStr">
         <ns0:is>
@@ -10531,6 +10228,9 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="J232" t="str" s="1">
+        <ns0:f>HYPERLINK("https://allensplumbinghi.com","allensplumbinghi.com")</ns0:f>
+      </ns0:c>
       <ns0:c r="K232" t="inlineStr">
         <ns0:is>
           <ns0:t>Google</ns0:t>
@@ -10573,10 +10273,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J233" t="inlineStr">
-        <ns0:is>
-          <ns0:t>bobthe.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J233" t="str" s="1">
+        <ns0:f>HYPERLINK("https://bobthe.com","bobthe.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K233" t="inlineStr">
         <ns0:is>
@@ -10620,10 +10318,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J234" t="inlineStr">
-        <ns0:is>
-          <ns0:t>larrystinson.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J234" t="str" s="1">
+        <ns0:f>HYPERLINK("https://larrystinson.com","larrystinson.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K234" t="inlineStr">
         <ns0:is>
@@ -10746,10 +10442,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J237" t="inlineStr">
-        <ns0:is>
-          <ns0:t>travisandsonsplumbing.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J237" t="str" s="1">
+        <ns0:f>HYPERLINK("https://travisandsonsplumbing.com","travisandsonsplumbing.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K237" t="inlineStr">
         <ns0:is>
@@ -10793,10 +10487,8 @@
           <ns0:t>YES</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="J238" t="inlineStr">
-        <ns0:is>
-          <ns0:t>southtexas.com</ns0:t>
-        </ns0:is>
+      <ns0:c r="J238" t="str" s="1">
+        <ns0:f>HYPERLINK("https://southtexas.com","southtexas.com")</ns0:f>
       </ns0:c>
       <ns0:c r="K238" t="inlineStr">
         <ns0:is>

</xml_diff>